<commit_message>
Apply user revised Filipino order and correct ten shifted drama codes
</commit_message>
<xml_diff>
--- a/schedules/filipino_20261105_20261115_two_daily/filipino_schedule_20261105_20261115.xlsx
+++ b/schedules/filipino_20261105_20261115_two_daily/filipino_schedule_20261105_20261115.xlsx
@@ -10,21 +10,23 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="每日两部总览" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="22条明细" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="跨频道7天核验" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="菲律宾语去重历史" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="合格片源与备选" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="文字禁播代运营排除" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="完整排片更新表" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="本次原表快照" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="排片说明" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10处代码校正" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="菲律宾语去重历史" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="合格片源与备选" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="文字禁播代运营排除" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="完整排片更新表" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="本次原表快照" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="排片说明" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'每日两部总览'!$A$1:$I$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'22条明细'!$A$1:$Q$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'跨频道7天核验'!$A$1:$F$23</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'菲律宾语去重历史'!$A$1:$C$37</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'合格片源与备选'!$A$1:$I$51</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'文字禁播代运营排除'!$A$1:$D$30</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'排片说明'!$A$1:$B$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'10处代码校正'!$A$1:$F$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'菲律宾语去重历史'!$A$1:$C$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'合格片源与备选'!$A$1:$I$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'文字禁播代运营排除'!$A$1:$D$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'排片说明'!$A$1:$B$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -534,12 +536,12 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>仙为仆，帝为奴，满宗弟子皆离谱</t>
+          <t>大明憨王爹我真想就藩</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2026 WW85</t>
+          <t>2026 WW73</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -564,7 +566,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>仙为仆，帝为奴，满宗弟子皆离谱/我在豪门装穷的日子</t>
+          <t>大明憨王爹我真想就藩/我在豪门装穷的日子</t>
         </is>
       </c>
     </row>
@@ -581,12 +583,12 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>叛出宗门后，我成了神级机甲师</t>
+          <t>七旬大爷每天买五斤鲜肉</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026 WW83</t>
+          <t>2026 WW71</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -611,7 +613,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>叛出宗门后，我成了神级机甲师/九世仙帝：王者归来</t>
+          <t>七旬大爷每天买五斤鲜肉/九世仙帝：王者归来</t>
         </is>
       </c>
     </row>
@@ -628,12 +630,12 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>车神归来：气运狂飙</t>
+          <t>龙鳞一响四海相护</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>2026 WW82</t>
+          <t>2026 WW69</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -658,7 +660,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>车神归来：气运狂飙/我仙途陨落，唯宠一人</t>
+          <t>龙鳞一响四海相护/我仙途陨落，唯宠一人</t>
         </is>
       </c>
     </row>
@@ -675,12 +677,12 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>闭关九年，魔女带娃找上门</t>
+          <t>分家开出海神的鱼钩</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2026 WW79</t>
+          <t>2026 WW67</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -705,7 +707,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>闭关九年，魔女带娃找上门/战神隐世：我的傲娇总裁表妹</t>
+          <t>分家开出海神的鱼钩/战神隐世：我的傲娇总裁表妹</t>
         </is>
       </c>
     </row>
@@ -722,12 +724,12 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>家庭煮夫竟是隐世总裁</t>
+          <t>全人类变小收录万灵的我无敌了</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2026 WW78</t>
+          <t>2026 WW65</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -752,7 +754,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>家庭煮夫竟是隐世总裁/娱乐圈凶神：我演反派就续命！</t>
+          <t>全人类变小收录万灵的我无敌了/娱乐圈凶神：我演反派就续命！</t>
         </is>
       </c>
     </row>
@@ -784,12 +786,12 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>大明憨王爹我真想就藩</t>
+          <t>仙为仆，帝为奴，满宗弟子皆离谱</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>2026 WW73</t>
+          <t>2026 WW85</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
@@ -799,7 +801,7 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>末日无限迷宫：开局设计精绝古城/大明憨王爹我真想就藩</t>
+          <t>末日无限迷宫：开局设计精绝古城/仙为仆，帝为奴，满宗弟子皆离谱</t>
         </is>
       </c>
     </row>
@@ -831,12 +833,12 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>七旬大爷每天买五斤鲜肉</t>
+          <t>叛出宗门后，我成了神级机甲师</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>2026 WW71</t>
+          <t>2026 WW83</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
@@ -846,7 +848,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>白月光被鱼钓走妻子悔断肠/七旬大爷每天买五斤鲜肉</t>
+          <t>白月光被鱼钓走妻子悔断肠/叛出宗门后，我成了神级机甲师</t>
         </is>
       </c>
     </row>
@@ -878,12 +880,12 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>龙鳞一响四海相护</t>
+          <t>车神归来：气运狂飙</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>2026 WW69</t>
+          <t>2026 WW82</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
@@ -893,7 +895,7 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>开局当牛照样养全家/龙鳞一响四海相护</t>
+          <t>开局当牛照样养全家/车神归来：气运狂飙</t>
         </is>
       </c>
     </row>
@@ -925,12 +927,12 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>分家开出海神的鱼钩</t>
+          <t>闭关九年，魔女带娃找上门</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>2026 WW67</t>
+          <t>2026 WW79</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
@@ -940,7 +942,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>天王之巨星归来/分家开出海神的鱼钩</t>
+          <t>天王之巨星归来/闭关九年，魔女带娃找上门</t>
         </is>
       </c>
     </row>
@@ -972,12 +974,12 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>全人类变小收录万灵的我无敌了</t>
+          <t>家庭煮夫竟是隐世总裁</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>2026 WW65</t>
+          <t>2026 WW78</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
@@ -987,7 +989,7 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>末日降临我的长工是丧尸/全人类变小收录万灵的我无敌了</t>
+          <t>末日降临我的长工是丧尸/家庭煮夫竟是隐世总裁</t>
         </is>
       </c>
     </row>
@@ -1040,6 +1042,169 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:I12"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>项目</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>说明</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="48" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>2026年10月30日修订</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>严格按用户最新表的剧名、日期与两档顺序调整；用户表10处剧名与代码错位，已按资源表修正。详见10处代码校正。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="48" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>范围与时间</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>2026年11月5—15日，每天北京时间12:00、17:00各一部，共22部；保留5部，新增17部。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="48" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>已有排片优先</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>以本次上传表为准；11月5—9日已有5部保留在原17:00档，11月5日前及其他频道剧目不动。此前已交付菲律宾语旧版排片只作保守去重，不覆盖本次表。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="48" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>空白表头</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>原表日期写到11月7日，后续空白表头按连续日期补到11月15日；菲律宾语原表后两部依次对应11月8日和9日，未移动剧目所在列。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="48" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>斜杠顺序</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>完整排片更新表菲律宾语行，每格“/”前为12:00，后为17:00；代表两部独立视频。原有剧留17:00。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="48" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>片源条件</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>最新资源表“最新剧集”：男频、菲律宾语标有或有/新；同剧任何版本文字标禁播或代运营则排除。按用户既定要求仅核验文字标记，不据颜色推断。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>2026年份依据</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>本次22部均为2026 WW代码片源，资源表未填明确出剧日期。仅确认代码标2026年，不将代码年份当作具体出剧日期或最新月份。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>外采解禁慢</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>11部标注“外采剧-解禁慢”，其中5部为原有安排、6部新增。未标禁播不代表已获版权放行，发布前按实际Studio版权状态核对；排期表已保留该状态。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>历史去重</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>新增17部与上传菲律宾语历史及此前已交付片单不重复；22部内部剧名和代码均无重复。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>同剧错峰</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>新增剧与本次其他频道表及已知未覆盖后续排片至少168小时；只给日期的按全天区间保守计算。命中无日期记录的候选不安排。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="48" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>交付范围</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>仅生成排片Excel、CSV和JSON，未修改线上飞书、YouTube或程序素材；未核验实际视频音轨。已有素材、标题和旧程序均不改。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1177,12 +1342,12 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>仙为仆，帝为奴，满宗弟子皆离谱</t>
+          <t>大明憨王爹我真想就藩</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2026 WW85</t>
+          <t>2026 WW73</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -1210,18 +1375,14 @@
           <t>有</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>外采剧-解禁慢</t>
-        </is>
-      </c>
+      <c r="K2" s="2" t="inlineStr"/>
       <c r="L2" s="2" t="inlineStr">
         <is>
           <t>最新剧集</t>
         </is>
       </c>
       <c r="M2" s="2" t="n">
-        <v>1132</v>
+        <v>1110</v>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
@@ -1339,12 +1500,12 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>叛出宗门后，我成了神级机甲师</t>
+          <t>七旬大爷每天买五斤鲜肉</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>2026 WW83</t>
+          <t>2026 WW71</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -1372,18 +1533,14 @@
           <t>有</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>外采剧-解禁慢</t>
-        </is>
-      </c>
+      <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr">
         <is>
           <t>最新剧集</t>
         </is>
       </c>
       <c r="M4" s="2" t="n">
-        <v>1130</v>
+        <v>1101</v>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
@@ -1501,12 +1658,12 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>车神归来：气运狂飙</t>
+          <t>龙鳞一响四海相护</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>2026 WW82</t>
+          <t>2026 WW69</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -1534,18 +1691,14 @@
           <t>有</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>外采剧-解禁慢</t>
-        </is>
-      </c>
+      <c r="K6" s="2" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr">
         <is>
           <t>最新剧集</t>
         </is>
       </c>
       <c r="M6" s="2" t="n">
-        <v>1128</v>
+        <v>1086</v>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
@@ -1663,12 +1816,12 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>闭关九年，魔女带娃找上门</t>
+          <t>分家开出海神的鱼钩</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>2026 WW79</t>
+          <t>2026 WW67</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -1696,23 +1849,17 @@
           <t>有</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>外采剧-解禁慢</t>
-        </is>
-      </c>
+      <c r="K8" s="2" t="inlineStr"/>
       <c r="L8" s="2" t="inlineStr">
         <is>
           <t>最新剧集</t>
         </is>
       </c>
       <c r="M8" s="2" t="n">
-        <v>1125</v>
-      </c>
-      <c r="N8" s="2" t="inlineStr">
-        <is>
-          <t>无同剧记录</t>
-        </is>
+        <v>1080</v>
+      </c>
+      <c r="N8" s="2" t="n">
+        <v>324</v>
       </c>
       <c r="O8" s="2" t="inlineStr"/>
       <c r="P8" s="2" t="inlineStr">
@@ -1829,12 +1976,12 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>家庭煮夫竟是隐世总裁</t>
+          <t>全人类变小收录万灵的我无敌了</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>2026 WW78</t>
+          <t>2026 WW65</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -1862,18 +2009,14 @@
           <t>有</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>外采剧-解禁慢</t>
-        </is>
-      </c>
+      <c r="K10" s="2" t="inlineStr"/>
       <c r="L10" s="2" t="inlineStr">
         <is>
           <t>最新剧集</t>
         </is>
       </c>
       <c r="M10" s="2" t="n">
-        <v>1124</v>
+        <v>1069</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
@@ -2076,12 +2219,12 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>大明憨王爹我真想就藩</t>
+          <t>仙为仆，帝为奴，满宗弟子皆离谱</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>2026 WW73</t>
+          <t>2026 WW85</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -2109,14 +2252,18 @@
           <t>有</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>外采剧-解禁慢</t>
+        </is>
+      </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
           <t>最新剧集</t>
         </is>
       </c>
       <c r="M13" s="2" t="n">
-        <v>1110</v>
+        <v>1132</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
@@ -2230,12 +2377,12 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>七旬大爷每天买五斤鲜肉</t>
+          <t>叛出宗门后，我成了神级机甲师</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>2026 WW71</t>
+          <t>2026 WW83</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
@@ -2263,14 +2410,18 @@
           <t>有</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>外采剧-解禁慢</t>
+        </is>
+      </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
           <t>最新剧集</t>
         </is>
       </c>
       <c r="M15" s="2" t="n">
-        <v>1101</v>
+        <v>1130</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
@@ -2384,12 +2535,12 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>龙鳞一响四海相护</t>
+          <t>车神归来：气运狂飙</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>2026 WW69</t>
+          <t>2026 WW82</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -2417,14 +2568,18 @@
           <t>有</t>
         </is>
       </c>
-      <c r="K17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>外采剧-解禁慢</t>
+        </is>
+      </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
           <t>最新剧集</t>
         </is>
       </c>
       <c r="M17" s="2" t="n">
-        <v>1086</v>
+        <v>1128</v>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
@@ -2538,12 +2693,12 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>分家开出海神的鱼钩</t>
+          <t>闭关九年，魔女带娃找上门</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>2026 WW67</t>
+          <t>2026 WW79</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
@@ -2571,17 +2726,23 @@
           <t>有</t>
         </is>
       </c>
-      <c r="K19" s="2" t="inlineStr"/>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>外采剧-解禁慢</t>
+        </is>
+      </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
           <t>最新剧集</t>
         </is>
       </c>
       <c r="M19" s="2" t="n">
-        <v>1080</v>
-      </c>
-      <c r="N19" s="2" t="n">
-        <v>449</v>
+        <v>1125</v>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>无同剧记录</t>
+        </is>
       </c>
       <c r="O19" s="2" t="inlineStr"/>
       <c r="P19" s="2" t="inlineStr">
@@ -2690,12 +2851,12 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>全人类变小收录万灵的我无敌了</t>
+          <t>家庭煮夫竟是隐世总裁</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>2026 WW65</t>
+          <t>2026 WW78</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
@@ -2723,14 +2884,18 @@
           <t>有</t>
         </is>
       </c>
-      <c r="K21" s="2" t="inlineStr"/>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>外采剧-解禁慢</t>
+        </is>
+      </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
           <t>最新剧集</t>
         </is>
       </c>
       <c r="M21" s="2" t="n">
-        <v>1069</v>
+        <v>1124</v>
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
@@ -2967,7 +3132,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>仙为仆，帝为奴，满宗弟子皆离谱</t>
+          <t>大明憨王爹我真想就藩</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -3031,7 +3196,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>叛出宗门后，我成了神级机甲师</t>
+          <t>七旬大爷每天买五斤鲜肉</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -3095,7 +3260,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>车神归来：气运狂飙</t>
+          <t>龙鳞一响四海相护</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -3159,7 +3324,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>闭关九年，魔女带娃找上门</t>
+          <t>分家开出海神的鱼钩</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -3174,7 +3339,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>无同剧记录</t>
+          <t>2026-10-25T00:00:00+08:00~2026-10-25T23:59:59.999999+08:00 英语2 本次最新排片表</t>
         </is>
       </c>
     </row>
@@ -3223,7 +3388,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>家庭煮夫竟是隐世总裁</t>
+          <t>全人类变小收录万灵的我无敌了</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -3319,7 +3484,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>大明憨王爹我真想就藩</t>
+          <t>仙为仆，帝为奴，满宗弟子皆离谱</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -3383,7 +3548,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>七旬大爷每天买五斤鲜肉</t>
+          <t>叛出宗门后，我成了神级机甲师</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -3447,7 +3612,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>龙鳞一响四海相护</t>
+          <t>车神归来：气运狂飙</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -3511,7 +3676,7 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>分家开出海神的鱼钩</t>
+          <t>闭关九年，魔女带娃找上门</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -3526,7 +3691,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25T00:00:00+08:00~2026-10-25T23:59:59.999999+08:00 英语2 本次最新排片表</t>
+          <t>无同剧记录</t>
         </is>
       </c>
     </row>
@@ -3575,7 +3740,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>全人类变小收录万灵的我无敌了</t>
+          <t>家庭煮夫竟是隐世总裁</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -3665,6 +3830,381 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>日期</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>北京时间</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>剧名</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>用户表所带代码</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>资源表正确代码</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>处理</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="48" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-05</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>大明憨王爹我真想就藩</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>2026 WW85</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>2026 WW73</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>按剧名匹配资源表修正代码</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="48" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-06</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>七旬大爷每天买五斤鲜肉</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>2026 WW83</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>2026 WW71</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>按剧名匹配资源表修正代码</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="48" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-07</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>龙鳞一响四海相护</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>2026 WW82</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>2026 WW69</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>按剧名匹配资源表修正代码</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="48" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-08</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>分家开出海神的鱼钩</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>2026 WW79</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>2026 WW67</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>按剧名匹配资源表修正代码</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="48" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-09</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>全人类变小收录万灵的我无敌了</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>2026 WW78</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>2026 WW65</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>按剧名匹配资源表修正代码</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="48" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>仙为仆，帝为奴，满宗弟子皆离谱</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>2026 WW73</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>2026 WW85</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>按剧名匹配资源表修正代码</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-11</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>叛出宗门后，我成了神级机甲师</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>2026 WW71</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>2026 WW83</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>按剧名匹配资源表修正代码</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-12</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>车神归来：气运狂飙</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>2026 WW69</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>2026 WW82</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>按剧名匹配资源表修正代码</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-13</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>闭关九年，魔女带娃找上门</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>2026 WW67</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>2026 WW79</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>按剧名匹配资源表修正代码</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-14</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>家庭煮夫竟是隐世总裁</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>2026 WW65</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>2026 WW78</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>按剧名匹配资源表修正代码</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F11"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4313,7 +4853,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6460,7 +7000,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7079,1624 +7619,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:D30"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:BJ8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="46" customWidth="1" min="3" max="3"/>
-    <col width="46" customWidth="1" min="4" max="4"/>
-    <col width="46" customWidth="1" min="5" max="5"/>
-    <col width="46" customWidth="1" min="6" max="6"/>
-    <col width="46" customWidth="1" min="7" max="7"/>
-    <col width="46" customWidth="1" min="8" max="8"/>
-    <col width="46" customWidth="1" min="9" max="9"/>
-    <col width="46" customWidth="1" min="10" max="10"/>
-    <col width="46" customWidth="1" min="11" max="11"/>
-    <col width="46" customWidth="1" min="12" max="12"/>
-    <col width="46" customWidth="1" min="13" max="13"/>
-    <col width="46" customWidth="1" min="14" max="14"/>
-    <col width="46" customWidth="1" min="15" max="15"/>
-    <col width="46" customWidth="1" min="16" max="16"/>
-    <col width="46" customWidth="1" min="17" max="17"/>
-    <col width="46" customWidth="1" min="18" max="18"/>
-    <col width="46" customWidth="1" min="19" max="19"/>
-    <col width="46" customWidth="1" min="20" max="20"/>
-    <col width="46" customWidth="1" min="21" max="21"/>
-    <col width="46" customWidth="1" min="22" max="22"/>
-    <col width="46" customWidth="1" min="23" max="23"/>
-    <col width="46" customWidth="1" min="24" max="24"/>
-    <col width="46" customWidth="1" min="25" max="25"/>
-    <col width="46" customWidth="1" min="26" max="26"/>
-    <col width="46" customWidth="1" min="27" max="27"/>
-    <col width="46" customWidth="1" min="28" max="28"/>
-    <col width="46" customWidth="1" min="29" max="29"/>
-    <col width="46" customWidth="1" min="30" max="30"/>
-    <col width="46" customWidth="1" min="31" max="31"/>
-    <col width="46" customWidth="1" min="32" max="32"/>
-    <col width="46" customWidth="1" min="33" max="33"/>
-    <col width="46" customWidth="1" min="34" max="34"/>
-    <col width="46" customWidth="1" min="35" max="35"/>
-    <col width="46" customWidth="1" min="36" max="36"/>
-    <col width="46" customWidth="1" min="37" max="37"/>
-    <col width="46" customWidth="1" min="38" max="38"/>
-    <col width="46" customWidth="1" min="39" max="39"/>
-    <col width="46" customWidth="1" min="40" max="40"/>
-    <col width="46" customWidth="1" min="41" max="41"/>
-    <col width="46" customWidth="1" min="42" max="42"/>
-    <col width="46" customWidth="1" min="43" max="43"/>
-    <col width="46" customWidth="1" min="44" max="44"/>
-    <col width="46" customWidth="1" min="45" max="45"/>
-    <col width="46" customWidth="1" min="46" max="46"/>
-    <col width="46" customWidth="1" min="47" max="47"/>
-    <col width="46" customWidth="1" min="48" max="48"/>
-    <col width="46" customWidth="1" min="49" max="49"/>
-    <col width="46" customWidth="1" min="50" max="50"/>
-    <col width="46" customWidth="1" min="51" max="51"/>
-    <col width="46" customWidth="1" min="52" max="52"/>
-    <col width="46" customWidth="1" min="53" max="53"/>
-    <col width="46" customWidth="1" min="54" max="54"/>
-    <col width="46" customWidth="1" min="55" max="55"/>
-    <col width="46" customWidth="1" min="56" max="56"/>
-    <col width="46" customWidth="1" min="57" max="57"/>
-    <col width="46" customWidth="1" min="58" max="58"/>
-    <col width="46" customWidth="1" min="59" max="59"/>
-    <col width="46" customWidth="1" min="60" max="60"/>
-    <col width="46" customWidth="1" min="61" max="61"/>
-    <col width="46" customWidth="1" min="62" max="62"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="25" customHeight="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>日期</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>2026.9.16</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>2026.9.17</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>2026.9.18</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>2026.9.19</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t>2026.9.20</t>
-        </is>
-      </c>
-      <c r="G1" s="2" t="inlineStr">
-        <is>
-          <t>2026.9.21</t>
-        </is>
-      </c>
-      <c r="H1" s="2" t="inlineStr">
-        <is>
-          <t>2026.9.22</t>
-        </is>
-      </c>
-      <c r="I1" s="2" t="inlineStr">
-        <is>
-          <t>2026.9.23</t>
-        </is>
-      </c>
-      <c r="J1" s="2" t="inlineStr">
-        <is>
-          <t>2026.9.24</t>
-        </is>
-      </c>
-      <c r="K1" s="2" t="inlineStr">
-        <is>
-          <t>2026.9.25</t>
-        </is>
-      </c>
-      <c r="L1" s="2" t="inlineStr">
-        <is>
-          <t>2026.9.26</t>
-        </is>
-      </c>
-      <c r="M1" s="2" t="inlineStr">
-        <is>
-          <t>2026.9.27</t>
-        </is>
-      </c>
-      <c r="N1" s="2" t="inlineStr">
-        <is>
-          <t>2026.9.28</t>
-        </is>
-      </c>
-      <c r="O1" s="2" t="inlineStr">
-        <is>
-          <t>2026.9.29</t>
-        </is>
-      </c>
-      <c r="P1" s="2" t="inlineStr">
-        <is>
-          <t>2026.9.30</t>
-        </is>
-      </c>
-      <c r="Q1" s="2" t="inlineStr">
-        <is>
-          <t>2026.10.1</t>
-        </is>
-      </c>
-      <c r="R1" s="2" t="inlineStr">
-        <is>
-          <t>2026.10.2</t>
-        </is>
-      </c>
-      <c r="S1" s="2" t="inlineStr">
-        <is>
-          <t>2026.10.3</t>
-        </is>
-      </c>
-      <c r="T1" s="2" t="inlineStr">
-        <is>
-          <t>2026.10.4</t>
-        </is>
-      </c>
-      <c r="U1" s="2" t="inlineStr">
-        <is>
-          <t>2026.10.5</t>
-        </is>
-      </c>
-      <c r="V1" s="2" t="inlineStr">
-        <is>
-          <t>2026.10.6</t>
-        </is>
-      </c>
-      <c r="W1" s="2" t="inlineStr">
-        <is>
-          <t>2026.10.7</t>
-        </is>
-      </c>
-      <c r="X1" s="2" t="inlineStr">
-        <is>
-          <t>2026.10.8</t>
-        </is>
-      </c>
-      <c r="Y1" s="2" t="inlineStr">
-        <is>
-          <t>2026.10.9</t>
-        </is>
-      </c>
-      <c r="Z1" s="2" t="inlineStr">
-        <is>
-          <t>2026.10.10</t>
-        </is>
-      </c>
-      <c r="AA1" s="2" t="inlineStr">
-        <is>
-          <t>2026.10.11</t>
-        </is>
-      </c>
-      <c r="AB1" s="2" t="inlineStr">
-        <is>
-          <t>2026.10.12</t>
-        </is>
-      </c>
-      <c r="AC1" s="2" t="inlineStr">
-        <is>
-          <t>2026.10.13</t>
-        </is>
-      </c>
-      <c r="AD1" s="2" t="inlineStr">
-        <is>
-          <t>2026.10.14</t>
-        </is>
-      </c>
-      <c r="AE1" s="2" t="inlineStr">
-        <is>
-          <t>2026.10.15</t>
-        </is>
-      </c>
-      <c r="AF1" s="2" t="inlineStr">
-        <is>
-          <t>2026.10.16</t>
-        </is>
-      </c>
-      <c r="AG1" s="2" t="inlineStr">
-        <is>
-          <t>2026.10.17</t>
-        </is>
-      </c>
-      <c r="AH1" s="2" t="inlineStr">
-        <is>
-          <t>2026.10.18</t>
-        </is>
-      </c>
-      <c r="AI1" s="2" t="inlineStr">
-        <is>
-          <t>2026.10.19</t>
-        </is>
-      </c>
-      <c r="AJ1" s="2" t="inlineStr">
-        <is>
-          <t>2026.10.20</t>
-        </is>
-      </c>
-      <c r="AK1" s="2" t="inlineStr">
-        <is>
-          <t>2026.10.21</t>
-        </is>
-      </c>
-      <c r="AL1" s="2" t="inlineStr">
-        <is>
-          <t>2026.10.22</t>
-        </is>
-      </c>
-      <c r="AM1" s="2" t="inlineStr">
-        <is>
-          <t>2026.10.23</t>
-        </is>
-      </c>
-      <c r="AN1" s="2" t="inlineStr">
-        <is>
-          <t>2026.10.24</t>
-        </is>
-      </c>
-      <c r="AO1" s="2" t="inlineStr">
-        <is>
-          <t>2026.10.25</t>
-        </is>
-      </c>
-      <c r="AP1" s="2" t="inlineStr">
-        <is>
-          <t>2026.10.26</t>
-        </is>
-      </c>
-      <c r="AQ1" s="2" t="inlineStr">
-        <is>
-          <t>2026.10.27</t>
-        </is>
-      </c>
-      <c r="AR1" s="2" t="inlineStr">
-        <is>
-          <t>2026.10.28</t>
-        </is>
-      </c>
-      <c r="AS1" s="2" t="inlineStr">
-        <is>
-          <t>2026.10.29</t>
-        </is>
-      </c>
-      <c r="AT1" s="2" t="inlineStr">
-        <is>
-          <t>2026.10.30</t>
-        </is>
-      </c>
-      <c r="AU1" s="2" t="inlineStr">
-        <is>
-          <t>2026.10.31</t>
-        </is>
-      </c>
-      <c r="AV1" s="2" t="inlineStr">
-        <is>
-          <t>2026.11.1</t>
-        </is>
-      </c>
-      <c r="AW1" s="2" t="inlineStr">
-        <is>
-          <t>2026.11.2</t>
-        </is>
-      </c>
-      <c r="AX1" s="2" t="inlineStr">
-        <is>
-          <t>2026.11.3</t>
-        </is>
-      </c>
-      <c r="AY1" s="2" t="inlineStr">
-        <is>
-          <t>2026.11.4</t>
-        </is>
-      </c>
-      <c r="AZ1" s="2" t="inlineStr">
-        <is>
-          <t>2026.11.5</t>
-        </is>
-      </c>
-      <c r="BA1" s="2" t="inlineStr">
-        <is>
-          <t>2026.11.6</t>
-        </is>
-      </c>
-      <c r="BB1" s="2" t="inlineStr">
-        <is>
-          <t>2026.11.7</t>
-        </is>
-      </c>
-      <c r="BC1" s="2" t="inlineStr">
-        <is>
-          <t>2026.11.8</t>
-        </is>
-      </c>
-      <c r="BD1" s="2" t="inlineStr">
-        <is>
-          <t>2026.11.9</t>
-        </is>
-      </c>
-      <c r="BE1" s="2" t="inlineStr">
-        <is>
-          <t>2026.11.10</t>
-        </is>
-      </c>
-      <c r="BF1" s="2" t="inlineStr">
-        <is>
-          <t>2026.11.11</t>
-        </is>
-      </c>
-      <c r="BG1" s="2" t="inlineStr">
-        <is>
-          <t>2026.11.12</t>
-        </is>
-      </c>
-      <c r="BH1" s="2" t="inlineStr">
-        <is>
-          <t>2026.11.13</t>
-        </is>
-      </c>
-      <c r="BI1" s="2" t="inlineStr">
-        <is>
-          <t>2026.11.14</t>
-        </is>
-      </c>
-      <c r="BJ1" s="2" t="inlineStr">
-        <is>
-          <t>2026.11.15</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="100" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>韩语</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>万道龙尊：开局把未婚妻扬了</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>我靠刷题重振宗门</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>大师兄竟是御兽宗宗主</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>开局上交系统我直升满级大佬</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>恐怖擂台我惊悚全世界</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>囤千万物资到古代娶女帝</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>玄孙女曝光我的仙人身份藏不住了</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>我的古井藏着大机缘</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>糟老头竟是剑仙</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>开局成破剑竟被她进化成神兵</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>诡异降临我召唤三千祖师反向入侵</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>我家浴缸通海底</t>
-        </is>
-      </c>
-      <c r="N2" s="2" t="inlineStr">
-        <is>
-          <t>武魂觉醒我用锤子一人成军</t>
-        </is>
-      </c>
-      <c r="O2" s="2" t="inlineStr">
-        <is>
-          <t>是谁坑惨了朕</t>
-        </is>
-      </c>
-      <c r="P2" s="2" t="inlineStr">
-        <is>
-          <t>燃香之后</t>
-        </is>
-      </c>
-      <c r="Q2" s="2" t="inlineStr">
-        <is>
-          <t>猴王报恩全村傻眼了</t>
-        </is>
-      </c>
-      <c r="R2" s="2" t="inlineStr">
-        <is>
-          <t>你退你的婚我撩我的师尊</t>
-        </is>
-      </c>
-      <c r="S2" s="2" t="inlineStr">
-        <is>
-          <t>我真是昏君你们快造反吧</t>
-        </is>
-      </c>
-      <c r="T2" s="2" t="inlineStr">
-        <is>
-          <t>我用科技征服人皇</t>
-        </is>
-      </c>
-      <c r="U2" s="2" t="inlineStr">
-        <is>
-          <t>我相亲捡属性开局怒怼化债女</t>
-        </is>
-      </c>
-      <c r="V2" s="2" t="inlineStr">
-        <is>
-          <t>夜闯病院-诡异幽影</t>
-        </is>
-      </c>
-      <c r="W2" s="2" t="inlineStr">
-        <is>
-          <t>热浪末世我带全家打造室外桃园</t>
-        </is>
-      </c>
-      <c r="X2" s="2" t="inlineStr">
-        <is>
-          <t>我在现代有个恐龙乐园</t>
-        </is>
-      </c>
-      <c r="Y2" s="2" t="inlineStr">
-        <is>
-          <t>上交修仙界</t>
-        </is>
-      </c>
-      <c r="Z2" s="2" t="inlineStr">
-        <is>
-          <t>开局流放我用系统搬空皇帝库房</t>
-        </is>
-      </c>
-      <c r="AA2" s="2" t="inlineStr">
-        <is>
-          <t>我造的机甲被老婆直播曝光了</t>
-        </is>
-      </c>
-      <c r="AB2" s="2" t="inlineStr">
-        <is>
-          <t>全界通缉我靠吞噬砍翻神明</t>
-        </is>
-      </c>
-      <c r="AC2" s="2" t="inlineStr">
-        <is>
-          <t>龙神报恩我一出海鱼获满满</t>
-        </is>
-      </c>
-      <c r="AD2" s="2" t="inlineStr">
-        <is>
-          <t>分家后我靠聚宝镯走上人生巅峰</t>
-        </is>
-      </c>
-      <c r="AE2" s="2" t="inlineStr">
-        <is>
-          <t>边疆老卒御赐老婆后我越活越勇</t>
-        </is>
-      </c>
-      <c r="AF2" s="2" t="inlineStr">
-        <is>
-          <t>寄生霸总我在死敌耳中低语</t>
-        </is>
-      </c>
-      <c r="AG2" s="2" t="inlineStr">
-        <is>
-          <t>让你当卧底谁让你成魔尊了</t>
-        </is>
-      </c>
-      <c r="AH2" s="2" t="inlineStr">
-        <is>
-          <t>真少爷他医术通神</t>
-        </is>
-      </c>
-      <c r="AI2" s="2" t="inlineStr">
-        <is>
-          <t>金丹冲进下水道貔貅丹道朝天啸</t>
-        </is>
-      </c>
-      <c r="AJ2" s="2" t="inlineStr">
-        <is>
-          <t>元始我申公豹请你上榜封神</t>
-        </is>
-      </c>
-      <c r="AK2" s="2" t="inlineStr">
-        <is>
-          <t>我的破烂牛棚堪比豪宅</t>
-        </is>
-      </c>
-      <c r="AL2" s="2" t="inlineStr">
-        <is>
-          <t>神级垂钓我钓尽世间天物</t>
-        </is>
-      </c>
-      <c r="AM2" s="2" t="inlineStr">
-        <is>
-          <t>SSS级狂龙横扫一切</t>
-        </is>
-      </c>
-      <c r="AN2" s="2" t="inlineStr">
-        <is>
-          <t>三年受尽凌辱，禁令解除我为龙主</t>
-        </is>
-      </c>
-      <c r="AO2" s="2" t="inlineStr">
-        <is>
-          <t>龙皇归来：不想当战神只要宠女儿</t>
-        </is>
-      </c>
-      <c r="AP2" s="2" t="inlineStr">
-        <is>
-          <t>代号枪神</t>
-        </is>
-      </c>
-      <c r="AQ2" s="2" t="inlineStr">
-        <is>
-          <t>《重回八零我靠山林奇珍系统养家》AI真人</t>
-        </is>
-      </c>
-      <c r="AR2" s="2" t="inlineStr">
-        <is>
-          <t>老年逆袭我竟成为山野之王</t>
-        </is>
-      </c>
-      <c r="AS2" s="2" t="inlineStr">
-        <is>
-          <t>山海计划我把整个修仙界上交了</t>
-        </is>
-      </c>
-      <c r="AT2" s="2" t="inlineStr">
-        <is>
-          <t>大爷俺踢球养活饥荒年全家</t>
-        </is>
-      </c>
-      <c r="AU2" s="2" t="inlineStr">
-        <is>
-          <t>空车超载还我三个亿的货</t>
-        </is>
-      </c>
-      <c r="AV2" s="2" t="inlineStr">
-        <is>
-          <t>奈何桥上不许刹车</t>
-        </is>
-      </c>
-      <c r="AW2" s="2" t="inlineStr">
-        <is>
-          <t>诡异擂台开局召唤左千户</t>
-        </is>
-      </c>
-      <c r="AX2" s="2" t="inlineStr">
-        <is>
-          <t>请祖宗出面讨公道</t>
-        </is>
-      </c>
-      <c r="AY2" s="2" t="inlineStr">
-        <is>
-          <t>不当黄牛全族发愁</t>
-        </is>
-      </c>
-      <c r="AZ2" s="2" t="inlineStr">
-        <is>
-          <t>九龙归位震八方</t>
-        </is>
-      </c>
-      <c r="BA2" s="2" t="inlineStr">
-        <is>
-          <t>自立门户干火锅，表哥急疯了</t>
-        </is>
-      </c>
-      <c r="BB2" s="2" t="inlineStr">
-        <is>
-          <t>不过一瓶醋</t>
-        </is>
-      </c>
-      <c r="BC2" s="2" t="inlineStr">
-        <is>
-          <t>归来后我踩碎所有偏见</t>
-        </is>
-      </c>
-      <c r="BD2" s="2" t="inlineStr">
-        <is>
-          <t>我宗门真的全是老弱病残啊</t>
-        </is>
-      </c>
-      <c r="BE2" s="2" t="inlineStr">
-        <is>
-          <t>只想种地扶贫奈何万民归顺</t>
-        </is>
-      </c>
-      <c r="BF2" s="2" t="inlineStr">
-        <is>
-          <t>旁人笑我木讷不知我有老仙金手指</t>
-        </is>
-      </c>
-      <c r="BG2" s="2" t="inlineStr">
-        <is>
-          <t>市井枭雄</t>
-        </is>
-      </c>
-      <c r="BH2" s="2" t="inlineStr">
-        <is>
-          <t>逆天纸扎铺</t>
-        </is>
-      </c>
-      <c r="BI2" s="2" t="inlineStr">
-        <is>
-          <t>穿越女频开局送皇后白月光进东厂</t>
-        </is>
-      </c>
-      <c r="BJ2" s="2" t="inlineStr">
-        <is>
-          <t>满级大师兄制霸都市</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="100" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>英语</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>SSS级狂龙横扫一切</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>三年受尽凌辱，禁令解除我为龙主</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>龙皇归来：不想当战神只要宠女儿</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>代号枪神</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>满级大师兄制霸都市</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>满朝文武都是我兄弟</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>开局流放我用系统搬空皇帝库房</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>是谁坑惨了朕</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>我真是昏君你们快造反吧</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>我用科技征服人皇</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>全球淹没我打造出了一座城池</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t>化身为树主宰万物</t>
-        </is>
-      </c>
-      <c r="N3" s="2" t="inlineStr">
-        <is>
-          <t>末日之我的房车无限升级</t>
-        </is>
-      </c>
-      <c r="O3" s="2" t="inlineStr">
-        <is>
-          <t>囤千万物资到古代娶女帝</t>
-        </is>
-      </c>
-      <c r="P3" s="2" t="inlineStr">
-        <is>
-          <t>开局成破剑竟被她进化成神兵</t>
-        </is>
-      </c>
-      <c r="Q3" s="2" t="inlineStr">
-        <is>
-          <t>流放开局，我卷走皇帝的小金库2</t>
-        </is>
-      </c>
-      <c r="R3" s="2" t="inlineStr">
-        <is>
-          <t>万道龙尊：开局把未婚妻扬了</t>
-        </is>
-      </c>
-      <c r="S3" s="2" t="inlineStr">
-        <is>
-          <t>恐怖擂台我惊悚全世界/高墙困恶邻</t>
-        </is>
-      </c>
-      <c r="T3" s="2" t="inlineStr">
-        <is>
-          <t>大师兄竟是御兽宗宗主</t>
-        </is>
-      </c>
-      <c r="U3" s="2" t="inlineStr">
-        <is>
-          <t>玄孙女曝光我的仙人身份藏不住了</t>
-        </is>
-      </c>
-      <c r="V3" s="2" t="inlineStr">
-        <is>
-          <t>绑定系统我在娱乐圈当教父</t>
-        </is>
-      </c>
-      <c r="W3" s="2" t="inlineStr">
-        <is>
-          <t>让你当卧底谁让你成魔尊了</t>
-        </is>
-      </c>
-      <c r="X3" s="2" t="inlineStr">
-        <is>
-          <t>朕的江山靠炮轰</t>
-        </is>
-      </c>
-      <c r="Y3" s="2" t="inlineStr">
-        <is>
-          <t>猴王报恩全村傻眼了/我带全村痛击大反派</t>
-        </is>
-      </c>
-      <c r="Z3" s="2" t="inlineStr">
-        <is>
-          <t>你退你的婚我撩我的师尊/全界通缉我靠吞噬砍翻神明</t>
-        </is>
-      </c>
-      <c r="AA3" s="2" t="inlineStr">
-        <is>
-          <t>九龙苏醒踏山河/瞎眼五百年我的学生全是三界大能</t>
-        </is>
-      </c>
-      <c r="AB3" s="2" t="inlineStr">
-        <is>
-          <t>诡异降临我召唤三千祖师反向入侵/全球竞速我的赛车能无限升级</t>
-        </is>
-      </c>
-      <c r="AC3" s="2" t="inlineStr">
-        <is>
-          <t>神级垂钓我钓尽世间天物/我在现代有个恐龙乐园</t>
-        </is>
-      </c>
-      <c r="AD3" s="2" t="inlineStr">
-        <is>
-          <t>我相亲捡属性开局怒怼化债女/边疆老卒御赐老婆后我越活越勇</t>
-        </is>
-      </c>
-      <c r="AE3" s="2" t="inlineStr">
-        <is>
-          <t>热浪末世我带全家打造室外桃园/我造的机甲被老婆直播曝光了</t>
-        </is>
-      </c>
-      <c r="AF3" s="2" t="inlineStr">
-        <is>
-          <t>上交修仙界/寄生霸总我在死敌耳中低语</t>
-        </is>
-      </c>
-      <c r="AG3" s="2" t="inlineStr">
-        <is>
-          <t>武魂觉醒我用锤子一人成军/一针定乾坤</t>
-        </is>
-      </c>
-      <c r="AH3" s="2" t="inlineStr">
-        <is>
-          <t>万倍返还弟子越强我越神/糟老头竟是剑仙</t>
-        </is>
-      </c>
-      <c r="AI3" s="2" t="inlineStr">
-        <is>
-          <t>让你木筏求生你度假娶老婆/全家穿越民国</t>
-        </is>
-      </c>
-      <c r="AJ3" s="2" t="inlineStr">
-        <is>
-          <t>我绑定亲情系统宠全家/我一邪修养反派为徒很正常吧</t>
-        </is>
-      </c>
-      <c r="AK3" s="2" t="inlineStr">
-        <is>
-          <t>同学会买单鱼头总对准我/九龙苏醒踏山河</t>
-        </is>
-      </c>
-      <c r="AL3" s="2" t="inlineStr">
-        <is>
-          <t>师娘送我出狱我横扫天下/太初神帝</t>
-        </is>
-      </c>
-      <c r="AM3" s="2" t="inlineStr">
-        <is>
-          <t>全球通缉：开局五星级越狱/纵横商海：被校花撞飞后，我苟成了世界首富</t>
-        </is>
-      </c>
-      <c r="AN3" s="2" t="inlineStr">
-        <is>
-          <t>被换灵骨后我成了大帝/满级枪神回都市开局领证</t>
-        </is>
-      </c>
-      <c r="AO3" s="2" t="inlineStr">
-        <is>
-          <t>我剑即天威/我的女友竟然是偶像歌手</t>
-        </is>
-      </c>
-      <c r="AP3" s="2" t="inlineStr"/>
-      <c r="AQ3" s="2" t="inlineStr"/>
-      <c r="AR3" s="2" t="inlineStr"/>
-      <c r="AS3" s="2" t="inlineStr"/>
-      <c r="AT3" s="2" t="inlineStr"/>
-      <c r="AU3" s="2" t="inlineStr"/>
-      <c r="AV3" s="2" t="inlineStr"/>
-      <c r="AW3" s="2" t="inlineStr"/>
-      <c r="AX3" s="2" t="inlineStr"/>
-      <c r="AY3" s="2" t="inlineStr"/>
-      <c r="AZ3" s="2" t="inlineStr"/>
-      <c r="BA3" s="2" t="inlineStr"/>
-      <c r="BB3" s="2" t="inlineStr"/>
-      <c r="BC3" s="2" t="inlineStr"/>
-      <c r="BD3" s="2" t="inlineStr"/>
-      <c r="BE3" s="2" t="inlineStr"/>
-      <c r="BF3" s="2" t="inlineStr"/>
-      <c r="BG3" s="2" t="inlineStr"/>
-      <c r="BH3" s="2" t="inlineStr"/>
-      <c r="BI3" s="2" t="inlineStr"/>
-      <c r="BJ3" s="2" t="inlineStr"/>
-    </row>
-    <row r="4" ht="100" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>西班牙</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr"/>
-      <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="2" t="inlineStr"/>
-      <c r="K4" s="2" t="inlineStr"/>
-      <c r="L4" s="2" t="inlineStr"/>
-      <c r="M4" s="2" t="inlineStr"/>
-      <c r="N4" s="2" t="inlineStr"/>
-      <c r="O4" s="2" t="inlineStr"/>
-      <c r="P4" s="2" t="inlineStr"/>
-      <c r="Q4" s="2" t="inlineStr">
-        <is>
-          <t>龙神医圣</t>
-        </is>
-      </c>
-      <c r="R4" s="2" t="inlineStr">
-        <is>
-          <t>重生千禧年我靠赶海带大哥致富</t>
-        </is>
-      </c>
-      <c r="S4" s="2" t="inlineStr">
-        <is>
-          <t>我的破烂牛棚堪比豪宅</t>
-        </is>
-      </c>
-      <c r="T4" s="2" t="inlineStr">
-        <is>
-          <t>龙神报恩我一出海鱼获满满</t>
-        </is>
-      </c>
-      <c r="U4" s="2" t="inlineStr">
-        <is>
-          <t>我造的机甲被老婆直播曝光了</t>
-        </is>
-      </c>
-      <c r="V4" s="2" t="inlineStr">
-        <is>
-          <t>元始我申公豹请你上榜封神</t>
-        </is>
-      </c>
-      <c r="W4" s="2" t="inlineStr">
-        <is>
-          <t>寄生霸总我在死敌耳中低语</t>
-        </is>
-      </c>
-      <c r="X4" s="2" t="inlineStr">
-        <is>
-          <t>奈何桥上不许刹车</t>
-        </is>
-      </c>
-      <c r="Y4" s="2" t="inlineStr">
-        <is>
-          <t>一箭定山河</t>
-        </is>
-      </c>
-      <c r="Z4" s="2" t="inlineStr">
-        <is>
-          <t>满朝文武都是我兄弟</t>
-        </is>
-      </c>
-      <c r="AA4" s="2" t="inlineStr">
-        <is>
-          <t>我用科技征服人皇</t>
-        </is>
-      </c>
-      <c r="AB4" s="2" t="inlineStr">
-        <is>
-          <t>是谁坑惨了朕</t>
-        </is>
-      </c>
-      <c r="AC4" s="2" t="inlineStr">
-        <is>
-          <t>SSS级狂龙横扫一切</t>
-        </is>
-      </c>
-      <c r="AD4" s="2" t="inlineStr">
-        <is>
-          <t>三年受尽凌辱，禁令解除我为龙主</t>
-        </is>
-      </c>
-      <c r="AE4" s="2" t="inlineStr">
-        <is>
-          <t>龙皇归来：不想当战神只要宠女儿</t>
-        </is>
-      </c>
-      <c r="AF4" s="2" t="inlineStr">
-        <is>
-          <t>开局流放我用系统搬空皇帝库房</t>
-        </is>
-      </c>
-      <c r="AG4" s="2" t="inlineStr">
-        <is>
-          <t>万道龙尊：开局把未婚妻扬了</t>
-        </is>
-      </c>
-      <c r="AH4" s="2" t="inlineStr">
-        <is>
-          <t>代号枪神</t>
-        </is>
-      </c>
-      <c r="AI4" s="2" t="inlineStr">
-        <is>
-          <t>我真是昏君你们快造反吧</t>
-        </is>
-      </c>
-      <c r="AJ4" s="2" t="inlineStr">
-        <is>
-          <t>末日之我的房车无限升级</t>
-        </is>
-      </c>
-      <c r="AK4" s="2" t="inlineStr">
-        <is>
-          <t>囤千万物资到古代娶女帝</t>
-        </is>
-      </c>
-      <c r="AL4" s="2" t="inlineStr">
-        <is>
-          <t>开局成破剑竟被她进化成神兵</t>
-        </is>
-      </c>
-      <c r="AM4" s="2" t="inlineStr">
-        <is>
-          <t>流放开局，我卷走皇帝的小金库2</t>
-        </is>
-      </c>
-      <c r="AN4" s="2" t="inlineStr">
-        <is>
-          <t>满级大师兄制霸都市</t>
-        </is>
-      </c>
-      <c r="AO4" s="2" t="inlineStr">
-        <is>
-          <t>归来后我踩碎所有偏见</t>
-        </is>
-      </c>
-      <c r="AP4" s="2" t="inlineStr"/>
-      <c r="AQ4" s="2" t="inlineStr"/>
-      <c r="AR4" s="2" t="inlineStr"/>
-      <c r="AS4" s="2" t="inlineStr"/>
-      <c r="AT4" s="2" t="inlineStr"/>
-      <c r="AU4" s="2" t="inlineStr"/>
-      <c r="AV4" s="2" t="inlineStr"/>
-      <c r="AW4" s="2" t="inlineStr"/>
-      <c r="AX4" s="2" t="inlineStr"/>
-      <c r="AY4" s="2" t="inlineStr"/>
-      <c r="AZ4" s="2" t="inlineStr"/>
-      <c r="BA4" s="2" t="inlineStr"/>
-      <c r="BB4" s="2" t="inlineStr"/>
-      <c r="BC4" s="2" t="inlineStr"/>
-      <c r="BD4" s="2" t="inlineStr"/>
-      <c r="BE4" s="2" t="inlineStr"/>
-      <c r="BF4" s="2" t="inlineStr"/>
-      <c r="BG4" s="2" t="inlineStr"/>
-      <c r="BH4" s="2" t="inlineStr"/>
-      <c r="BI4" s="2" t="inlineStr"/>
-      <c r="BJ4" s="2" t="inlineStr"/>
-    </row>
-    <row r="5" ht="140" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>菲律宾</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr"/>
-      <c r="C5" s="2" t="inlineStr"/>
-      <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr"/>
-      <c r="I5" s="2" t="inlineStr"/>
-      <c r="J5" s="2" t="inlineStr"/>
-      <c r="K5" s="2" t="inlineStr"/>
-      <c r="L5" s="2" t="inlineStr"/>
-      <c r="M5" s="2" t="inlineStr"/>
-      <c r="N5" s="2" t="inlineStr"/>
-      <c r="O5" s="2" t="inlineStr"/>
-      <c r="P5" s="2" t="inlineStr"/>
-      <c r="Q5" s="2" t="inlineStr"/>
-      <c r="R5" s="2" t="inlineStr"/>
-      <c r="S5" s="2" t="inlineStr"/>
-      <c r="T5" s="2" t="inlineStr"/>
-      <c r="U5" s="2" t="inlineStr"/>
-      <c r="V5" s="2" t="inlineStr"/>
-      <c r="W5" s="2" t="inlineStr"/>
-      <c r="X5" s="2" t="inlineStr"/>
-      <c r="Y5" s="2" t="inlineStr"/>
-      <c r="Z5" s="2" t="inlineStr"/>
-      <c r="AA5" s="2" t="inlineStr"/>
-      <c r="AB5" s="2" t="inlineStr"/>
-      <c r="AC5" s="2" t="inlineStr"/>
-      <c r="AD5" s="2" t="inlineStr"/>
-      <c r="AE5" s="2" t="inlineStr"/>
-      <c r="AF5" s="2" t="inlineStr">
-        <is>
-          <t>玄孙女曝光我的仙人身份藏不住了</t>
-        </is>
-      </c>
-      <c r="AG5" s="2" t="inlineStr">
-        <is>
-          <t>全球淹没我打造出了一座城池</t>
-        </is>
-      </c>
-      <c r="AH5" s="2" t="inlineStr">
-        <is>
-          <t>我家浴缸通海底</t>
-        </is>
-      </c>
-      <c r="AI5" s="2" t="inlineStr">
-        <is>
-          <t>分家后我靠聚宝镯走上人生巅峰</t>
-        </is>
-      </c>
-      <c r="AJ5" s="2" t="inlineStr">
-        <is>
-          <t>九龙归位震八方</t>
-        </is>
-      </c>
-      <c r="AK5" s="2" t="inlineStr">
-        <is>
-          <t>我相亲捡属性开局怒怼化债女</t>
-        </is>
-      </c>
-      <c r="AL5" s="2" t="inlineStr">
-        <is>
-          <t>满级枪神回都市开局领证</t>
-        </is>
-      </c>
-      <c r="AM5" s="2" t="inlineStr">
-        <is>
-          <t>全民荒原求生</t>
-        </is>
-      </c>
-      <c r="AN5" s="2" t="inlineStr">
-        <is>
-          <t>万古第一仙在都市</t>
-        </is>
-      </c>
-      <c r="AO5" s="2" t="inlineStr">
-        <is>
-          <t>水库无限加速钓鱼佬排队爆杆</t>
-        </is>
-      </c>
-      <c r="AP5" s="2" t="inlineStr">
-        <is>
-          <t>战神归来前妻你哭什么</t>
-        </is>
-      </c>
-      <c r="AQ5" s="2" t="inlineStr">
-        <is>
-          <t>旁人笑我木讷不知我有老仙金手指</t>
-        </is>
-      </c>
-      <c r="AR5" s="2" t="inlineStr">
-        <is>
-          <t>婚礼照常新娘换人</t>
-        </is>
-      </c>
-      <c r="AS5" s="2" t="inlineStr">
-        <is>
-          <t>穿越女频开局送皇后白月光进东厂</t>
-        </is>
-      </c>
-      <c r="AT5" s="2" t="inlineStr">
-        <is>
-          <t>龙神报恩我一出海鱼获满满</t>
-        </is>
-      </c>
-      <c r="AU5" s="2" t="inlineStr"/>
-      <c r="AV5" s="2" t="inlineStr"/>
-      <c r="AW5" s="2" t="inlineStr"/>
-      <c r="AX5" s="2" t="inlineStr"/>
-      <c r="AY5" s="2" t="inlineStr"/>
-      <c r="AZ5" s="2" t="inlineStr">
-        <is>
-          <t>仙为仆，帝为奴，满宗弟子皆离谱/我在豪门装穷的日子</t>
-        </is>
-      </c>
-      <c r="BA5" s="2" t="inlineStr">
-        <is>
-          <t>叛出宗门后，我成了神级机甲师/九世仙帝：王者归来</t>
-        </is>
-      </c>
-      <c r="BB5" s="2" t="inlineStr">
-        <is>
-          <t>车神归来：气运狂飙/我仙途陨落，唯宠一人</t>
-        </is>
-      </c>
-      <c r="BC5" s="2" t="inlineStr">
-        <is>
-          <t>闭关九年，魔女带娃找上门/战神隐世：我的傲娇总裁表妹</t>
-        </is>
-      </c>
-      <c r="BD5" s="2" t="inlineStr">
-        <is>
-          <t>家庭煮夫竟是隐世总裁/娱乐圈凶神：我演反派就续命！</t>
-        </is>
-      </c>
-      <c r="BE5" s="2" t="inlineStr">
-        <is>
-          <t>末日无限迷宫：开局设计精绝古城/大明憨王爹我真想就藩</t>
-        </is>
-      </c>
-      <c r="BF5" s="2" t="inlineStr">
-        <is>
-          <t>白月光被鱼钓走妻子悔断肠/七旬大爷每天买五斤鲜肉</t>
-        </is>
-      </c>
-      <c r="BG5" s="2" t="inlineStr">
-        <is>
-          <t>开局当牛照样养全家/龙鳞一响四海相护</t>
-        </is>
-      </c>
-      <c r="BH5" s="2" t="inlineStr">
-        <is>
-          <t>天王之巨星归来/分家开出海神的鱼钩</t>
-        </is>
-      </c>
-      <c r="BI5" s="2" t="inlineStr">
-        <is>
-          <t>末日降临我的长工是丧尸/全人类变小收录万灵的我无敌了</t>
-        </is>
-      </c>
-      <c r="BJ5" s="2" t="inlineStr">
-        <is>
-          <t>神临我自执剑迎/重回八零我靠山林奇珍系统养家</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="100" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>俄语男频</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr"/>
-      <c r="C6" s="2" t="inlineStr"/>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr"/>
-      <c r="I6" s="2" t="inlineStr"/>
-      <c r="J6" s="2" t="inlineStr"/>
-      <c r="K6" s="2" t="inlineStr"/>
-      <c r="L6" s="2" t="inlineStr"/>
-      <c r="M6" s="2" t="inlineStr"/>
-      <c r="N6" s="2" t="inlineStr"/>
-      <c r="O6" s="2" t="inlineStr"/>
-      <c r="P6" s="2" t="inlineStr"/>
-      <c r="Q6" s="2" t="inlineStr"/>
-      <c r="R6" s="2" t="inlineStr"/>
-      <c r="S6" s="2" t="inlineStr"/>
-      <c r="T6" s="2" t="inlineStr"/>
-      <c r="U6" s="2" t="inlineStr"/>
-      <c r="V6" s="2" t="inlineStr"/>
-      <c r="W6" s="2" t="inlineStr"/>
-      <c r="X6" s="2" t="inlineStr"/>
-      <c r="Y6" s="2" t="inlineStr"/>
-      <c r="Z6" s="2" t="inlineStr"/>
-      <c r="AA6" s="2" t="inlineStr"/>
-      <c r="AB6" s="2" t="inlineStr"/>
-      <c r="AC6" s="2" t="inlineStr"/>
-      <c r="AD6" s="2" t="inlineStr"/>
-      <c r="AE6" s="2" t="inlineStr"/>
-      <c r="AF6" s="2" t="inlineStr"/>
-      <c r="AG6" s="2" t="inlineStr"/>
-      <c r="AH6" s="2" t="inlineStr"/>
-      <c r="AI6" s="2" t="inlineStr"/>
-      <c r="AJ6" s="2" t="inlineStr">
-        <is>
-          <t>边疆老卒御赐老婆后我越活越勇</t>
-        </is>
-      </c>
-      <c r="AK6" s="2" t="inlineStr">
-        <is>
-          <t>我宗门真的全是老弱病残啊</t>
-        </is>
-      </c>
-      <c r="AL6" s="2" t="inlineStr">
-        <is>
-          <t>我靠医术横扫江都</t>
-        </is>
-      </c>
-      <c r="AM6" s="2" t="inlineStr">
-        <is>
-          <t>武魂觉醒我用锤子一人成军</t>
-        </is>
-      </c>
-      <c r="AN6" s="2" t="inlineStr">
-        <is>
-          <t>九龙归位震八方</t>
-        </is>
-      </c>
-      <c r="AO6" s="2" t="inlineStr">
-        <is>
-          <t>分家后我靠聚宝镯走上人生巅峰</t>
-        </is>
-      </c>
-      <c r="AP6" s="2" t="inlineStr">
-        <is>
-          <t>我相亲捡属性开局怒怼化债女</t>
-        </is>
-      </c>
-      <c r="AQ6" s="2" t="inlineStr">
-        <is>
-          <t>归来后我踩碎所有偏见</t>
-        </is>
-      </c>
-      <c r="AR6" s="2" t="inlineStr">
-        <is>
-          <t>战神归来前妻你哭什么</t>
-        </is>
-      </c>
-      <c r="AS6" s="2" t="inlineStr">
-        <is>
-          <t>旁人笑我木讷不知我有老仙金手指</t>
-        </is>
-      </c>
-      <c r="AT6" s="2" t="inlineStr">
-        <is>
-          <t>婚礼照常新娘换人</t>
-        </is>
-      </c>
-      <c r="AU6" s="2" t="inlineStr">
-        <is>
-          <t>穿越女频开局送皇后白月光进东厂</t>
-        </is>
-      </c>
-      <c r="AV6" s="2" t="inlineStr">
-        <is>
-          <t>龙神报恩我一出海鱼获满满</t>
-        </is>
-      </c>
-      <c r="AW6" s="2" t="inlineStr">
-        <is>
-          <t>我造的机甲被老婆直播曝光了</t>
-        </is>
-      </c>
-      <c r="AX6" s="2" t="inlineStr">
-        <is>
-          <t>猴王报恩全村傻眼了</t>
-        </is>
-      </c>
-      <c r="AY6" s="2" t="inlineStr">
-        <is>
-          <t>我家浴缸通海底</t>
-        </is>
-      </c>
-      <c r="AZ6" s="2" t="inlineStr">
-        <is>
-          <t>玄孙女曝光我的仙人身份藏不住了</t>
-        </is>
-      </c>
-      <c r="BA6" s="2" t="inlineStr">
-        <is>
-          <t>渔夫从神奇龙珠开始起飞</t>
-        </is>
-      </c>
-      <c r="BB6" s="2" t="inlineStr">
-        <is>
-          <t>万倍返还弟子越强我越神</t>
-        </is>
-      </c>
-      <c r="BC6" s="2" t="inlineStr">
-        <is>
-          <t>满级大师兄制霸都市</t>
-        </is>
-      </c>
-      <c r="BD6" s="2" t="inlineStr">
-        <is>
-          <t>囤千万物资到古代娶女帝</t>
-        </is>
-      </c>
-      <c r="BE6" s="2" t="inlineStr">
-        <is>
-          <t>跌入古井觉醒神农秘术</t>
-        </is>
-      </c>
-      <c r="BF6" s="2" t="inlineStr"/>
-      <c r="BG6" s="2" t="inlineStr"/>
-      <c r="BH6" s="2" t="inlineStr"/>
-      <c r="BI6" s="2" t="inlineStr"/>
-      <c r="BJ6" s="2" t="inlineStr"/>
-    </row>
-    <row r="7" ht="100" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>英语男频2</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr"/>
-      <c r="C7" s="2" t="inlineStr"/>
-      <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr"/>
-      <c r="I7" s="2" t="inlineStr"/>
-      <c r="J7" s="2" t="inlineStr"/>
-      <c r="K7" s="2" t="inlineStr"/>
-      <c r="L7" s="2" t="inlineStr"/>
-      <c r="M7" s="2" t="inlineStr"/>
-      <c r="N7" s="2" t="inlineStr"/>
-      <c r="O7" s="2" t="inlineStr"/>
-      <c r="P7" s="2" t="inlineStr"/>
-      <c r="Q7" s="2" t="inlineStr"/>
-      <c r="R7" s="2" t="inlineStr"/>
-      <c r="S7" s="2" t="inlineStr"/>
-      <c r="T7" s="2" t="inlineStr"/>
-      <c r="U7" s="2" t="inlineStr"/>
-      <c r="V7" s="2" t="inlineStr"/>
-      <c r="W7" s="2" t="inlineStr"/>
-      <c r="X7" s="2" t="inlineStr"/>
-      <c r="Y7" s="2" t="inlineStr"/>
-      <c r="Z7" s="2" t="inlineStr"/>
-      <c r="AA7" s="2" t="inlineStr"/>
-      <c r="AB7" s="2" t="inlineStr"/>
-      <c r="AC7" s="2" t="inlineStr"/>
-      <c r="AD7" s="2" t="inlineStr"/>
-      <c r="AE7" s="2" t="inlineStr"/>
-      <c r="AF7" s="2" t="inlineStr"/>
-      <c r="AG7" s="2" t="inlineStr"/>
-      <c r="AH7" s="2" t="inlineStr"/>
-      <c r="AI7" s="2" t="inlineStr"/>
-      <c r="AJ7" s="2" t="inlineStr"/>
-      <c r="AK7" s="2" t="inlineStr"/>
-      <c r="AL7" s="2" t="inlineStr"/>
-      <c r="AM7" s="2" t="inlineStr"/>
-      <c r="AN7" s="2" t="inlineStr">
-        <is>
-          <t>神临我自执剑迎</t>
-        </is>
-      </c>
-      <c r="AO7" s="2" t="inlineStr">
-        <is>
-          <t>分家开出海神的鱼钩</t>
-        </is>
-      </c>
-      <c r="AP7" s="2" t="inlineStr">
-        <is>
-          <t>满级大师兄制霸都市</t>
-        </is>
-      </c>
-      <c r="AQ7" s="2" t="inlineStr">
-        <is>
-          <t>满朝文武都是我兄弟</t>
-        </is>
-      </c>
-      <c r="AR7" s="2" t="inlineStr">
-        <is>
-          <t>开局流放我用系统搬空皇帝库房</t>
-        </is>
-      </c>
-      <c r="AS7" s="2" t="inlineStr">
-        <is>
-          <t>是谁坑惨了朕</t>
-        </is>
-      </c>
-      <c r="AT7" s="2" t="inlineStr">
-        <is>
-          <t>我真是昏君你们快造反吧</t>
-        </is>
-      </c>
-      <c r="AU7" s="2" t="inlineStr">
-        <is>
-          <t>我用科技征服人皇</t>
-        </is>
-      </c>
-      <c r="AV7" s="2" t="inlineStr">
-        <is>
-          <t>全球淹没我打造出了一座城池</t>
-        </is>
-      </c>
-      <c r="AW7" s="2" t="inlineStr">
-        <is>
-          <t>囤千万物资到古代娶女帝</t>
-        </is>
-      </c>
-      <c r="AX7" s="2" t="inlineStr">
-        <is>
-          <t>龙皇归来：不想当战神只要宠女儿</t>
-        </is>
-      </c>
-      <c r="AY7" s="2" t="inlineStr">
-        <is>
-          <t>流放开局，我卷走皇帝的小金库2</t>
-        </is>
-      </c>
-      <c r="AZ7" s="2" t="inlineStr">
-        <is>
-          <t>开局成破剑竟被她进化成神兵</t>
-        </is>
-      </c>
-      <c r="BA7" s="2" t="inlineStr">
-        <is>
-          <t>代号枪神</t>
-        </is>
-      </c>
-      <c r="BB7" s="2" t="inlineStr"/>
-      <c r="BC7" s="2" t="inlineStr"/>
-      <c r="BD7" s="2" t="inlineStr"/>
-      <c r="BE7" s="2" t="inlineStr"/>
-      <c r="BF7" s="2" t="inlineStr"/>
-      <c r="BG7" s="2" t="inlineStr"/>
-      <c r="BH7" s="2" t="inlineStr"/>
-      <c r="BI7" s="2" t="inlineStr"/>
-      <c r="BJ7" s="2" t="inlineStr"/>
-    </row>
-    <row r="8" ht="100" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>（注：部分内容由豆包工作 AI 生成）</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr"/>
-      <c r="C8" s="2" t="inlineStr"/>
-      <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr"/>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr"/>
-      <c r="I8" s="2" t="inlineStr"/>
-      <c r="J8" s="2" t="inlineStr"/>
-      <c r="K8" s="2" t="inlineStr"/>
-      <c r="L8" s="2" t="inlineStr"/>
-      <c r="M8" s="2" t="inlineStr"/>
-      <c r="N8" s="2" t="inlineStr"/>
-      <c r="O8" s="2" t="inlineStr"/>
-      <c r="P8" s="2" t="inlineStr"/>
-      <c r="Q8" s="2" t="inlineStr"/>
-      <c r="R8" s="2" t="inlineStr"/>
-      <c r="S8" s="2" t="inlineStr"/>
-      <c r="T8" s="2" t="inlineStr"/>
-      <c r="U8" s="2" t="inlineStr"/>
-      <c r="V8" s="2" t="inlineStr"/>
-      <c r="W8" s="2" t="inlineStr"/>
-      <c r="X8" s="2" t="inlineStr"/>
-      <c r="Y8" s="2" t="inlineStr"/>
-      <c r="Z8" s="2" t="inlineStr"/>
-      <c r="AA8" s="2" t="inlineStr"/>
-      <c r="AB8" s="2" t="inlineStr"/>
-      <c r="AC8" s="2" t="inlineStr"/>
-      <c r="AD8" s="2" t="inlineStr"/>
-      <c r="AE8" s="2" t="inlineStr"/>
-      <c r="AF8" s="2" t="inlineStr"/>
-      <c r="AG8" s="2" t="inlineStr"/>
-      <c r="AH8" s="2" t="inlineStr"/>
-      <c r="AI8" s="2" t="inlineStr"/>
-      <c r="AJ8" s="2" t="inlineStr"/>
-      <c r="AK8" s="2" t="inlineStr"/>
-      <c r="AL8" s="2" t="inlineStr"/>
-      <c r="AM8" s="2" t="inlineStr"/>
-      <c r="AN8" s="2" t="inlineStr"/>
-      <c r="AO8" s="2" t="inlineStr"/>
-      <c r="AP8" s="2" t="inlineStr"/>
-      <c r="AQ8" s="2" t="inlineStr"/>
-      <c r="AR8" s="2" t="inlineStr"/>
-      <c r="AS8" s="2" t="inlineStr"/>
-      <c r="AT8" s="2" t="inlineStr"/>
-      <c r="AU8" s="2" t="inlineStr"/>
-      <c r="AV8" s="2" t="inlineStr"/>
-      <c r="AW8" s="2" t="inlineStr"/>
-      <c r="AX8" s="2" t="inlineStr"/>
-      <c r="AY8" s="2" t="inlineStr"/>
-      <c r="AZ8" s="2" t="inlineStr"/>
-      <c r="BA8" s="2" t="inlineStr"/>
-      <c r="BB8" s="2" t="inlineStr"/>
-      <c r="BC8" s="2" t="inlineStr"/>
-      <c r="BD8" s="2" t="inlineStr"/>
-      <c r="BE8" s="2" t="inlineStr"/>
-      <c r="BF8" s="2" t="inlineStr"/>
-      <c r="BG8" s="2" t="inlineStr"/>
-      <c r="BH8" s="2" t="inlineStr"/>
-      <c r="BI8" s="2" t="inlineStr"/>
-      <c r="BJ8" s="2" t="inlineStr"/>
-    </row>
-  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9045,14 +7967,46 @@
           <t>2026.11.7</t>
         </is>
       </c>
-      <c r="BC1" s="2" t="inlineStr"/>
-      <c r="BD1" s="2" t="inlineStr"/>
-      <c r="BE1" s="2" t="inlineStr"/>
-      <c r="BF1" s="2" t="inlineStr"/>
-      <c r="BG1" s="2" t="inlineStr"/>
-      <c r="BH1" s="2" t="inlineStr"/>
-      <c r="BI1" s="2" t="inlineStr"/>
-      <c r="BJ1" s="2" t="inlineStr"/>
+      <c r="BC1" s="2" t="inlineStr">
+        <is>
+          <t>2026.11.8</t>
+        </is>
+      </c>
+      <c r="BD1" s="2" t="inlineStr">
+        <is>
+          <t>2026.11.9</t>
+        </is>
+      </c>
+      <c r="BE1" s="2" t="inlineStr">
+        <is>
+          <t>2026.11.10</t>
+        </is>
+      </c>
+      <c r="BF1" s="2" t="inlineStr">
+        <is>
+          <t>2026.11.11</t>
+        </is>
+      </c>
+      <c r="BG1" s="2" t="inlineStr">
+        <is>
+          <t>2026.11.12</t>
+        </is>
+      </c>
+      <c r="BH1" s="2" t="inlineStr">
+        <is>
+          <t>2026.11.13</t>
+        </is>
+      </c>
+      <c r="BI1" s="2" t="inlineStr">
+        <is>
+          <t>2026.11.14</t>
+        </is>
+      </c>
+      <c r="BJ1" s="2" t="inlineStr">
+        <is>
+          <t>2026.11.15</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="100" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -9880,35 +8834,59 @@
       <c r="AY5" s="2" t="inlineStr"/>
       <c r="AZ5" s="2" t="inlineStr">
         <is>
-          <t>我在豪门装穷的日子/</t>
+          <t>大明憨王爹我真想就藩/我在豪门装穷的日子</t>
         </is>
       </c>
       <c r="BA5" s="2" t="inlineStr">
         <is>
-          <t>九世仙帝：王者归来</t>
+          <t>七旬大爷每天买五斤鲜肉/九世仙帝：王者归来</t>
         </is>
       </c>
       <c r="BB5" s="2" t="inlineStr">
         <is>
-          <t>我仙途陨落，唯宠一人</t>
+          <t>龙鳞一响四海相护/我仙途陨落，唯宠一人</t>
         </is>
       </c>
       <c r="BC5" s="2" t="inlineStr">
         <is>
-          <t>战神隐世：我的傲娇总裁表妹</t>
+          <t>分家开出海神的鱼钩/战神隐世：我的傲娇总裁表妹</t>
         </is>
       </c>
       <c r="BD5" s="2" t="inlineStr">
         <is>
-          <t>娱乐圈凶神：我演反派就续命！</t>
-        </is>
-      </c>
-      <c r="BE5" s="2" t="inlineStr"/>
-      <c r="BF5" s="2" t="inlineStr"/>
-      <c r="BG5" s="2" t="inlineStr"/>
-      <c r="BH5" s="2" t="inlineStr"/>
-      <c r="BI5" s="2" t="inlineStr"/>
-      <c r="BJ5" s="2" t="inlineStr"/>
+          <t>全人类变小收录万灵的我无敌了/娱乐圈凶神：我演反派就续命！</t>
+        </is>
+      </c>
+      <c r="BE5" s="2" t="inlineStr">
+        <is>
+          <t>末日无限迷宫：开局设计精绝古城/仙为仆，帝为奴，满宗弟子皆离谱</t>
+        </is>
+      </c>
+      <c r="BF5" s="2" t="inlineStr">
+        <is>
+          <t>白月光被鱼钓走妻子悔断肠/叛出宗门后，我成了神级机甲师</t>
+        </is>
+      </c>
+      <c r="BG5" s="2" t="inlineStr">
+        <is>
+          <t>开局当牛照样养全家/车神归来：气运狂飙</t>
+        </is>
+      </c>
+      <c r="BH5" s="2" t="inlineStr">
+        <is>
+          <t>天王之巨星归来/闭关九年，魔女带娃找上门</t>
+        </is>
+      </c>
+      <c r="BI5" s="2" t="inlineStr">
+        <is>
+          <t>末日降临我的长工是丧尸/家庭煮夫竟是隐世总裁</t>
+        </is>
+      </c>
+      <c r="BJ5" s="2" t="inlineStr">
+        <is>
+          <t>神临我自执剑迎/重回八零我靠山林奇珍系统养家</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="100" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -10269,147 +9247,1558 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:BJ8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="110" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
+    <col width="46" customWidth="1" min="7" max="7"/>
+    <col width="46" customWidth="1" min="8" max="8"/>
+    <col width="46" customWidth="1" min="9" max="9"/>
+    <col width="46" customWidth="1" min="10" max="10"/>
+    <col width="46" customWidth="1" min="11" max="11"/>
+    <col width="46" customWidth="1" min="12" max="12"/>
+    <col width="46" customWidth="1" min="13" max="13"/>
+    <col width="46" customWidth="1" min="14" max="14"/>
+    <col width="46" customWidth="1" min="15" max="15"/>
+    <col width="46" customWidth="1" min="16" max="16"/>
+    <col width="46" customWidth="1" min="17" max="17"/>
+    <col width="46" customWidth="1" min="18" max="18"/>
+    <col width="46" customWidth="1" min="19" max="19"/>
+    <col width="46" customWidth="1" min="20" max="20"/>
+    <col width="46" customWidth="1" min="21" max="21"/>
+    <col width="46" customWidth="1" min="22" max="22"/>
+    <col width="46" customWidth="1" min="23" max="23"/>
+    <col width="46" customWidth="1" min="24" max="24"/>
+    <col width="46" customWidth="1" min="25" max="25"/>
+    <col width="46" customWidth="1" min="26" max="26"/>
+    <col width="46" customWidth="1" min="27" max="27"/>
+    <col width="46" customWidth="1" min="28" max="28"/>
+    <col width="46" customWidth="1" min="29" max="29"/>
+    <col width="46" customWidth="1" min="30" max="30"/>
+    <col width="46" customWidth="1" min="31" max="31"/>
+    <col width="46" customWidth="1" min="32" max="32"/>
+    <col width="46" customWidth="1" min="33" max="33"/>
+    <col width="46" customWidth="1" min="34" max="34"/>
+    <col width="46" customWidth="1" min="35" max="35"/>
+    <col width="46" customWidth="1" min="36" max="36"/>
+    <col width="46" customWidth="1" min="37" max="37"/>
+    <col width="46" customWidth="1" min="38" max="38"/>
+    <col width="46" customWidth="1" min="39" max="39"/>
+    <col width="46" customWidth="1" min="40" max="40"/>
+    <col width="46" customWidth="1" min="41" max="41"/>
+    <col width="46" customWidth="1" min="42" max="42"/>
+    <col width="46" customWidth="1" min="43" max="43"/>
+    <col width="46" customWidth="1" min="44" max="44"/>
+    <col width="46" customWidth="1" min="45" max="45"/>
+    <col width="46" customWidth="1" min="46" max="46"/>
+    <col width="46" customWidth="1" min="47" max="47"/>
+    <col width="46" customWidth="1" min="48" max="48"/>
+    <col width="46" customWidth="1" min="49" max="49"/>
+    <col width="46" customWidth="1" min="50" max="50"/>
+    <col width="46" customWidth="1" min="51" max="51"/>
+    <col width="46" customWidth="1" min="52" max="52"/>
+    <col width="46" customWidth="1" min="53" max="53"/>
+    <col width="46" customWidth="1" min="54" max="54"/>
+    <col width="46" customWidth="1" min="55" max="55"/>
+    <col width="46" customWidth="1" min="56" max="56"/>
+    <col width="46" customWidth="1" min="57" max="57"/>
+    <col width="46" customWidth="1" min="58" max="58"/>
+    <col width="46" customWidth="1" min="59" max="59"/>
+    <col width="46" customWidth="1" min="60" max="60"/>
+    <col width="46" customWidth="1" min="61" max="61"/>
+    <col width="46" customWidth="1" min="62" max="62"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>项目</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>说明</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="48" customHeight="1">
+    <row r="1" ht="25" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>日期</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>2026.9.16</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>2026.9.17</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>2026.9.18</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>2026.9.19</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>2026.9.20</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>2026.9.21</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>2026.9.22</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>2026.9.23</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>2026.9.24</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>2026.9.25</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>2026.9.26</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>2026.9.27</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>2026.9.28</t>
+        </is>
+      </c>
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>2026.9.29</t>
+        </is>
+      </c>
+      <c r="P1" s="2" t="inlineStr">
+        <is>
+          <t>2026.9.30</t>
+        </is>
+      </c>
+      <c r="Q1" s="2" t="inlineStr">
+        <is>
+          <t>2026.10.1</t>
+        </is>
+      </c>
+      <c r="R1" s="2" t="inlineStr">
+        <is>
+          <t>2026.10.2</t>
+        </is>
+      </c>
+      <c r="S1" s="2" t="inlineStr">
+        <is>
+          <t>2026.10.3</t>
+        </is>
+      </c>
+      <c r="T1" s="2" t="inlineStr">
+        <is>
+          <t>2026.10.4</t>
+        </is>
+      </c>
+      <c r="U1" s="2" t="inlineStr">
+        <is>
+          <t>2026.10.5</t>
+        </is>
+      </c>
+      <c r="V1" s="2" t="inlineStr">
+        <is>
+          <t>2026.10.6</t>
+        </is>
+      </c>
+      <c r="W1" s="2" t="inlineStr">
+        <is>
+          <t>2026.10.7</t>
+        </is>
+      </c>
+      <c r="X1" s="2" t="inlineStr">
+        <is>
+          <t>2026.10.8</t>
+        </is>
+      </c>
+      <c r="Y1" s="2" t="inlineStr">
+        <is>
+          <t>2026.10.9</t>
+        </is>
+      </c>
+      <c r="Z1" s="2" t="inlineStr">
+        <is>
+          <t>2026.10.10</t>
+        </is>
+      </c>
+      <c r="AA1" s="2" t="inlineStr">
+        <is>
+          <t>2026.10.11</t>
+        </is>
+      </c>
+      <c r="AB1" s="2" t="inlineStr">
+        <is>
+          <t>2026.10.12</t>
+        </is>
+      </c>
+      <c r="AC1" s="2" t="inlineStr">
+        <is>
+          <t>2026.10.13</t>
+        </is>
+      </c>
+      <c r="AD1" s="2" t="inlineStr">
+        <is>
+          <t>2026.10.14</t>
+        </is>
+      </c>
+      <c r="AE1" s="2" t="inlineStr">
+        <is>
+          <t>2026.10.15</t>
+        </is>
+      </c>
+      <c r="AF1" s="2" t="inlineStr">
+        <is>
+          <t>2026.10.16</t>
+        </is>
+      </c>
+      <c r="AG1" s="2" t="inlineStr">
+        <is>
+          <t>2026.10.17</t>
+        </is>
+      </c>
+      <c r="AH1" s="2" t="inlineStr">
+        <is>
+          <t>2026.10.18</t>
+        </is>
+      </c>
+      <c r="AI1" s="2" t="inlineStr">
+        <is>
+          <t>2026.10.19</t>
+        </is>
+      </c>
+      <c r="AJ1" s="2" t="inlineStr">
+        <is>
+          <t>2026.10.20</t>
+        </is>
+      </c>
+      <c r="AK1" s="2" t="inlineStr">
+        <is>
+          <t>2026.10.21</t>
+        </is>
+      </c>
+      <c r="AL1" s="2" t="inlineStr">
+        <is>
+          <t>2026.10.22</t>
+        </is>
+      </c>
+      <c r="AM1" s="2" t="inlineStr">
+        <is>
+          <t>2026.10.23</t>
+        </is>
+      </c>
+      <c r="AN1" s="2" t="inlineStr">
+        <is>
+          <t>2026.10.24</t>
+        </is>
+      </c>
+      <c r="AO1" s="2" t="inlineStr">
+        <is>
+          <t>2026.10.25</t>
+        </is>
+      </c>
+      <c r="AP1" s="2" t="inlineStr">
+        <is>
+          <t>2026.10.26</t>
+        </is>
+      </c>
+      <c r="AQ1" s="2" t="inlineStr">
+        <is>
+          <t>2026.10.27</t>
+        </is>
+      </c>
+      <c r="AR1" s="2" t="inlineStr">
+        <is>
+          <t>2026.10.28</t>
+        </is>
+      </c>
+      <c r="AS1" s="2" t="inlineStr">
+        <is>
+          <t>2026.10.29</t>
+        </is>
+      </c>
+      <c r="AT1" s="2" t="inlineStr">
+        <is>
+          <t>2026.10.30</t>
+        </is>
+      </c>
+      <c r="AU1" s="2" t="inlineStr">
+        <is>
+          <t>2026.10.31</t>
+        </is>
+      </c>
+      <c r="AV1" s="2" t="inlineStr">
+        <is>
+          <t>2026.11.1</t>
+        </is>
+      </c>
+      <c r="AW1" s="2" t="inlineStr">
+        <is>
+          <t>2026.11.2</t>
+        </is>
+      </c>
+      <c r="AX1" s="2" t="inlineStr">
+        <is>
+          <t>2026.11.3</t>
+        </is>
+      </c>
+      <c r="AY1" s="2" t="inlineStr">
+        <is>
+          <t>2026.11.4</t>
+        </is>
+      </c>
+      <c r="AZ1" s="2" t="inlineStr">
+        <is>
+          <t>2026.11.5</t>
+        </is>
+      </c>
+      <c r="BA1" s="2" t="inlineStr">
+        <is>
+          <t>2026.11.6</t>
+        </is>
+      </c>
+      <c r="BB1" s="2" t="inlineStr">
+        <is>
+          <t>2026.11.7</t>
+        </is>
+      </c>
+      <c r="BC1" s="2" t="inlineStr"/>
+      <c r="BD1" s="2" t="inlineStr"/>
+      <c r="BE1" s="2" t="inlineStr"/>
+      <c r="BF1" s="2" t="inlineStr"/>
+      <c r="BG1" s="2" t="inlineStr"/>
+      <c r="BH1" s="2" t="inlineStr"/>
+      <c r="BI1" s="2" t="inlineStr"/>
+      <c r="BJ1" s="2" t="inlineStr"/>
+    </row>
+    <row r="2" ht="100" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>范围与时间</t>
+          <t>韩语</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026年11月5—15日，每天北京时间12:00、17:00各一部，共22部；保留5部，新增17部。</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="48" customHeight="1">
+          <t>万道龙尊：开局把未婚妻扬了</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>我靠刷题重振宗门</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>大师兄竟是御兽宗宗主</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>开局上交系统我直升满级大佬</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>恐怖擂台我惊悚全世界</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>囤千万物资到古代娶女帝</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>玄孙女曝光我的仙人身份藏不住了</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>我的古井藏着大机缘</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>糟老头竟是剑仙</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>开局成破剑竟被她进化成神兵</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>诡异降临我召唤三千祖师反向入侵</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>我家浴缸通海底</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>武魂觉醒我用锤子一人成军</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>是谁坑惨了朕</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>燃香之后</t>
+        </is>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>猴王报恩全村傻眼了</t>
+        </is>
+      </c>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
+          <t>你退你的婚我撩我的师尊</t>
+        </is>
+      </c>
+      <c r="S2" s="2" t="inlineStr">
+        <is>
+          <t>我真是昏君你们快造反吧</t>
+        </is>
+      </c>
+      <c r="T2" s="2" t="inlineStr">
+        <is>
+          <t>我用科技征服人皇</t>
+        </is>
+      </c>
+      <c r="U2" s="2" t="inlineStr">
+        <is>
+          <t>我相亲捡属性开局怒怼化债女</t>
+        </is>
+      </c>
+      <c r="V2" s="2" t="inlineStr">
+        <is>
+          <t>夜闯病院-诡异幽影</t>
+        </is>
+      </c>
+      <c r="W2" s="2" t="inlineStr">
+        <is>
+          <t>热浪末世我带全家打造室外桃园</t>
+        </is>
+      </c>
+      <c r="X2" s="2" t="inlineStr">
+        <is>
+          <t>我在现代有个恐龙乐园</t>
+        </is>
+      </c>
+      <c r="Y2" s="2" t="inlineStr">
+        <is>
+          <t>上交修仙界</t>
+        </is>
+      </c>
+      <c r="Z2" s="2" t="inlineStr">
+        <is>
+          <t>开局流放我用系统搬空皇帝库房</t>
+        </is>
+      </c>
+      <c r="AA2" s="2" t="inlineStr">
+        <is>
+          <t>我造的机甲被老婆直播曝光了</t>
+        </is>
+      </c>
+      <c r="AB2" s="2" t="inlineStr">
+        <is>
+          <t>全界通缉我靠吞噬砍翻神明</t>
+        </is>
+      </c>
+      <c r="AC2" s="2" t="inlineStr">
+        <is>
+          <t>龙神报恩我一出海鱼获满满</t>
+        </is>
+      </c>
+      <c r="AD2" s="2" t="inlineStr">
+        <is>
+          <t>分家后我靠聚宝镯走上人生巅峰</t>
+        </is>
+      </c>
+      <c r="AE2" s="2" t="inlineStr">
+        <is>
+          <t>边疆老卒御赐老婆后我越活越勇</t>
+        </is>
+      </c>
+      <c r="AF2" s="2" t="inlineStr">
+        <is>
+          <t>寄生霸总我在死敌耳中低语</t>
+        </is>
+      </c>
+      <c r="AG2" s="2" t="inlineStr">
+        <is>
+          <t>让你当卧底谁让你成魔尊了</t>
+        </is>
+      </c>
+      <c r="AH2" s="2" t="inlineStr">
+        <is>
+          <t>真少爷他医术通神</t>
+        </is>
+      </c>
+      <c r="AI2" s="2" t="inlineStr">
+        <is>
+          <t>金丹冲进下水道貔貅丹道朝天啸</t>
+        </is>
+      </c>
+      <c r="AJ2" s="2" t="inlineStr">
+        <is>
+          <t>元始我申公豹请你上榜封神</t>
+        </is>
+      </c>
+      <c r="AK2" s="2" t="inlineStr">
+        <is>
+          <t>我的破烂牛棚堪比豪宅</t>
+        </is>
+      </c>
+      <c r="AL2" s="2" t="inlineStr">
+        <is>
+          <t>神级垂钓我钓尽世间天物</t>
+        </is>
+      </c>
+      <c r="AM2" s="2" t="inlineStr">
+        <is>
+          <t>SSS级狂龙横扫一切</t>
+        </is>
+      </c>
+      <c r="AN2" s="2" t="inlineStr">
+        <is>
+          <t>三年受尽凌辱，禁令解除我为龙主</t>
+        </is>
+      </c>
+      <c r="AO2" s="2" t="inlineStr">
+        <is>
+          <t>龙皇归来：不想当战神只要宠女儿</t>
+        </is>
+      </c>
+      <c r="AP2" s="2" t="inlineStr">
+        <is>
+          <t>代号枪神</t>
+        </is>
+      </c>
+      <c r="AQ2" s="2" t="inlineStr">
+        <is>
+          <t>《重回八零我靠山林奇珍系统养家》AI真人</t>
+        </is>
+      </c>
+      <c r="AR2" s="2" t="inlineStr">
+        <is>
+          <t>老年逆袭我竟成为山野之王</t>
+        </is>
+      </c>
+      <c r="AS2" s="2" t="inlineStr">
+        <is>
+          <t>山海计划我把整个修仙界上交了</t>
+        </is>
+      </c>
+      <c r="AT2" s="2" t="inlineStr">
+        <is>
+          <t>大爷俺踢球养活饥荒年全家</t>
+        </is>
+      </c>
+      <c r="AU2" s="2" t="inlineStr">
+        <is>
+          <t>空车超载还我三个亿的货</t>
+        </is>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>奈何桥上不许刹车</t>
+        </is>
+      </c>
+      <c r="AW2" s="2" t="inlineStr">
+        <is>
+          <t>诡异擂台开局召唤左千户</t>
+        </is>
+      </c>
+      <c r="AX2" s="2" t="inlineStr">
+        <is>
+          <t>请祖宗出面讨公道</t>
+        </is>
+      </c>
+      <c r="AY2" s="2" t="inlineStr">
+        <is>
+          <t>不当黄牛全族发愁</t>
+        </is>
+      </c>
+      <c r="AZ2" s="2" t="inlineStr">
+        <is>
+          <t>九龙归位震八方</t>
+        </is>
+      </c>
+      <c r="BA2" s="2" t="inlineStr">
+        <is>
+          <t>自立门户干火锅，表哥急疯了</t>
+        </is>
+      </c>
+      <c r="BB2" s="2" t="inlineStr">
+        <is>
+          <t>不过一瓶醋</t>
+        </is>
+      </c>
+      <c r="BC2" s="2" t="inlineStr">
+        <is>
+          <t>归来后我踩碎所有偏见</t>
+        </is>
+      </c>
+      <c r="BD2" s="2" t="inlineStr">
+        <is>
+          <t>我宗门真的全是老弱病残啊</t>
+        </is>
+      </c>
+      <c r="BE2" s="2" t="inlineStr">
+        <is>
+          <t>只想种地扶贫奈何万民归顺</t>
+        </is>
+      </c>
+      <c r="BF2" s="2" t="inlineStr">
+        <is>
+          <t>旁人笑我木讷不知我有老仙金手指</t>
+        </is>
+      </c>
+      <c r="BG2" s="2" t="inlineStr">
+        <is>
+          <t>市井枭雄</t>
+        </is>
+      </c>
+      <c r="BH2" s="2" t="inlineStr">
+        <is>
+          <t>逆天纸扎铺</t>
+        </is>
+      </c>
+      <c r="BI2" s="2" t="inlineStr">
+        <is>
+          <t>穿越女频开局送皇后白月光进东厂</t>
+        </is>
+      </c>
+      <c r="BJ2" s="2" t="inlineStr">
+        <is>
+          <t>满级大师兄制霸都市</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="100" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>已有排片优先</t>
+          <t>英语</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>以本次上传表为准；11月5—9日已有5部保留在原17:00档，11月5日前及其他频道剧目不动。此前已交付菲律宾语旧版排片只作保守去重，不覆盖本次表。</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="48" customHeight="1">
+          <t>SSS级狂龙横扫一切</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>三年受尽凌辱，禁令解除我为龙主</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>龙皇归来：不想当战神只要宠女儿</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>代号枪神</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>满级大师兄制霸都市</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>满朝文武都是我兄弟</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>开局流放我用系统搬空皇帝库房</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>是谁坑惨了朕</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>我真是昏君你们快造反吧</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>我用科技征服人皇</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>全球淹没我打造出了一座城池</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>化身为树主宰万物</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>末日之我的房车无限升级</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>囤千万物资到古代娶女帝</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>开局成破剑竟被她进化成神兵</t>
+        </is>
+      </c>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>流放开局，我卷走皇帝的小金库2</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>万道龙尊：开局把未婚妻扬了</t>
+        </is>
+      </c>
+      <c r="S3" s="2" t="inlineStr">
+        <is>
+          <t>恐怖擂台我惊悚全世界/高墙困恶邻</t>
+        </is>
+      </c>
+      <c r="T3" s="2" t="inlineStr">
+        <is>
+          <t>大师兄竟是御兽宗宗主</t>
+        </is>
+      </c>
+      <c r="U3" s="2" t="inlineStr">
+        <is>
+          <t>玄孙女曝光我的仙人身份藏不住了</t>
+        </is>
+      </c>
+      <c r="V3" s="2" t="inlineStr">
+        <is>
+          <t>绑定系统我在娱乐圈当教父</t>
+        </is>
+      </c>
+      <c r="W3" s="2" t="inlineStr">
+        <is>
+          <t>让你当卧底谁让你成魔尊了</t>
+        </is>
+      </c>
+      <c r="X3" s="2" t="inlineStr">
+        <is>
+          <t>朕的江山靠炮轰</t>
+        </is>
+      </c>
+      <c r="Y3" s="2" t="inlineStr">
+        <is>
+          <t>猴王报恩全村傻眼了/我带全村痛击大反派</t>
+        </is>
+      </c>
+      <c r="Z3" s="2" t="inlineStr">
+        <is>
+          <t>你退你的婚我撩我的师尊/全界通缉我靠吞噬砍翻神明</t>
+        </is>
+      </c>
+      <c r="AA3" s="2" t="inlineStr">
+        <is>
+          <t>九龙苏醒踏山河/瞎眼五百年我的学生全是三界大能</t>
+        </is>
+      </c>
+      <c r="AB3" s="2" t="inlineStr">
+        <is>
+          <t>诡异降临我召唤三千祖师反向入侵/全球竞速我的赛车能无限升级</t>
+        </is>
+      </c>
+      <c r="AC3" s="2" t="inlineStr">
+        <is>
+          <t>神级垂钓我钓尽世间天物/我在现代有个恐龙乐园</t>
+        </is>
+      </c>
+      <c r="AD3" s="2" t="inlineStr">
+        <is>
+          <t>我相亲捡属性开局怒怼化债女/边疆老卒御赐老婆后我越活越勇</t>
+        </is>
+      </c>
+      <c r="AE3" s="2" t="inlineStr">
+        <is>
+          <t>热浪末世我带全家打造室外桃园/我造的机甲被老婆直播曝光了</t>
+        </is>
+      </c>
+      <c r="AF3" s="2" t="inlineStr">
+        <is>
+          <t>上交修仙界/寄生霸总我在死敌耳中低语</t>
+        </is>
+      </c>
+      <c r="AG3" s="2" t="inlineStr">
+        <is>
+          <t>武魂觉醒我用锤子一人成军/一针定乾坤</t>
+        </is>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>万倍返还弟子越强我越神/糟老头竟是剑仙</t>
+        </is>
+      </c>
+      <c r="AI3" s="2" t="inlineStr">
+        <is>
+          <t>让你木筏求生你度假娶老婆/全家穿越民国</t>
+        </is>
+      </c>
+      <c r="AJ3" s="2" t="inlineStr">
+        <is>
+          <t>我绑定亲情系统宠全家/我一邪修养反派为徒很正常吧</t>
+        </is>
+      </c>
+      <c r="AK3" s="2" t="inlineStr">
+        <is>
+          <t>同学会买单鱼头总对准我/九龙苏醒踏山河</t>
+        </is>
+      </c>
+      <c r="AL3" s="2" t="inlineStr">
+        <is>
+          <t>师娘送我出狱我横扫天下/太初神帝</t>
+        </is>
+      </c>
+      <c r="AM3" s="2" t="inlineStr">
+        <is>
+          <t>全球通缉：开局五星级越狱/纵横商海：被校花撞飞后，我苟成了世界首富</t>
+        </is>
+      </c>
+      <c r="AN3" s="2" t="inlineStr">
+        <is>
+          <t>被换灵骨后我成了大帝/满级枪神回都市开局领证</t>
+        </is>
+      </c>
+      <c r="AO3" s="2" t="inlineStr">
+        <is>
+          <t>我剑即天威/我的女友竟然是偶像歌手</t>
+        </is>
+      </c>
+      <c r="AP3" s="2" t="inlineStr"/>
+      <c r="AQ3" s="2" t="inlineStr"/>
+      <c r="AR3" s="2" t="inlineStr"/>
+      <c r="AS3" s="2" t="inlineStr"/>
+      <c r="AT3" s="2" t="inlineStr"/>
+      <c r="AU3" s="2" t="inlineStr"/>
+      <c r="AV3" s="2" t="inlineStr"/>
+      <c r="AW3" s="2" t="inlineStr"/>
+      <c r="AX3" s="2" t="inlineStr"/>
+      <c r="AY3" s="2" t="inlineStr"/>
+      <c r="AZ3" s="2" t="inlineStr"/>
+      <c r="BA3" s="2" t="inlineStr"/>
+      <c r="BB3" s="2" t="inlineStr"/>
+      <c r="BC3" s="2" t="inlineStr"/>
+      <c r="BD3" s="2" t="inlineStr"/>
+      <c r="BE3" s="2" t="inlineStr"/>
+      <c r="BF3" s="2" t="inlineStr"/>
+      <c r="BG3" s="2" t="inlineStr"/>
+      <c r="BH3" s="2" t="inlineStr"/>
+      <c r="BI3" s="2" t="inlineStr"/>
+      <c r="BJ3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4" ht="100" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>空白表头</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>原表日期写到11月7日，后续空白表头按连续日期补到11月15日；菲律宾语原表后两部依次对应11月8日和9日，未移动剧目所在列。</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="48" customHeight="1">
+          <t>西班牙</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr"/>
+      <c r="N4" s="2" t="inlineStr"/>
+      <c r="O4" s="2" t="inlineStr"/>
+      <c r="P4" s="2" t="inlineStr"/>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>龙神医圣</t>
+        </is>
+      </c>
+      <c r="R4" s="2" t="inlineStr">
+        <is>
+          <t>重生千禧年我靠赶海带大哥致富</t>
+        </is>
+      </c>
+      <c r="S4" s="2" t="inlineStr">
+        <is>
+          <t>我的破烂牛棚堪比豪宅</t>
+        </is>
+      </c>
+      <c r="T4" s="2" t="inlineStr">
+        <is>
+          <t>龙神报恩我一出海鱼获满满</t>
+        </is>
+      </c>
+      <c r="U4" s="2" t="inlineStr">
+        <is>
+          <t>我造的机甲被老婆直播曝光了</t>
+        </is>
+      </c>
+      <c r="V4" s="2" t="inlineStr">
+        <is>
+          <t>元始我申公豹请你上榜封神</t>
+        </is>
+      </c>
+      <c r="W4" s="2" t="inlineStr">
+        <is>
+          <t>寄生霸总我在死敌耳中低语</t>
+        </is>
+      </c>
+      <c r="X4" s="2" t="inlineStr">
+        <is>
+          <t>奈何桥上不许刹车</t>
+        </is>
+      </c>
+      <c r="Y4" s="2" t="inlineStr">
+        <is>
+          <t>一箭定山河</t>
+        </is>
+      </c>
+      <c r="Z4" s="2" t="inlineStr">
+        <is>
+          <t>满朝文武都是我兄弟</t>
+        </is>
+      </c>
+      <c r="AA4" s="2" t="inlineStr">
+        <is>
+          <t>我用科技征服人皇</t>
+        </is>
+      </c>
+      <c r="AB4" s="2" t="inlineStr">
+        <is>
+          <t>是谁坑惨了朕</t>
+        </is>
+      </c>
+      <c r="AC4" s="2" t="inlineStr">
+        <is>
+          <t>SSS级狂龙横扫一切</t>
+        </is>
+      </c>
+      <c r="AD4" s="2" t="inlineStr">
+        <is>
+          <t>三年受尽凌辱，禁令解除我为龙主</t>
+        </is>
+      </c>
+      <c r="AE4" s="2" t="inlineStr">
+        <is>
+          <t>龙皇归来：不想当战神只要宠女儿</t>
+        </is>
+      </c>
+      <c r="AF4" s="2" t="inlineStr">
+        <is>
+          <t>开局流放我用系统搬空皇帝库房</t>
+        </is>
+      </c>
+      <c r="AG4" s="2" t="inlineStr">
+        <is>
+          <t>万道龙尊：开局把未婚妻扬了</t>
+        </is>
+      </c>
+      <c r="AH4" s="2" t="inlineStr">
+        <is>
+          <t>代号枪神</t>
+        </is>
+      </c>
+      <c r="AI4" s="2" t="inlineStr">
+        <is>
+          <t>我真是昏君你们快造反吧</t>
+        </is>
+      </c>
+      <c r="AJ4" s="2" t="inlineStr">
+        <is>
+          <t>末日之我的房车无限升级</t>
+        </is>
+      </c>
+      <c r="AK4" s="2" t="inlineStr">
+        <is>
+          <t>囤千万物资到古代娶女帝</t>
+        </is>
+      </c>
+      <c r="AL4" s="2" t="inlineStr">
+        <is>
+          <t>开局成破剑竟被她进化成神兵</t>
+        </is>
+      </c>
+      <c r="AM4" s="2" t="inlineStr">
+        <is>
+          <t>流放开局，我卷走皇帝的小金库2</t>
+        </is>
+      </c>
+      <c r="AN4" s="2" t="inlineStr">
+        <is>
+          <t>满级大师兄制霸都市</t>
+        </is>
+      </c>
+      <c r="AO4" s="2" t="inlineStr">
+        <is>
+          <t>归来后我踩碎所有偏见</t>
+        </is>
+      </c>
+      <c r="AP4" s="2" t="inlineStr"/>
+      <c r="AQ4" s="2" t="inlineStr"/>
+      <c r="AR4" s="2" t="inlineStr"/>
+      <c r="AS4" s="2" t="inlineStr"/>
+      <c r="AT4" s="2" t="inlineStr"/>
+      <c r="AU4" s="2" t="inlineStr"/>
+      <c r="AV4" s="2" t="inlineStr"/>
+      <c r="AW4" s="2" t="inlineStr"/>
+      <c r="AX4" s="2" t="inlineStr"/>
+      <c r="AY4" s="2" t="inlineStr"/>
+      <c r="AZ4" s="2" t="inlineStr"/>
+      <c r="BA4" s="2" t="inlineStr"/>
+      <c r="BB4" s="2" t="inlineStr"/>
+      <c r="BC4" s="2" t="inlineStr"/>
+      <c r="BD4" s="2" t="inlineStr"/>
+      <c r="BE4" s="2" t="inlineStr"/>
+      <c r="BF4" s="2" t="inlineStr"/>
+      <c r="BG4" s="2" t="inlineStr"/>
+      <c r="BH4" s="2" t="inlineStr"/>
+      <c r="BI4" s="2" t="inlineStr"/>
+      <c r="BJ4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5" ht="140" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>斜杠顺序</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>完整排片更新表菲律宾语行，每格“/”前为12:00，后为17:00；代表两部独立视频。原有剧留17:00。</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="48" customHeight="1">
+          <t>菲律宾</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr"/>
+      <c r="D5" s="2" t="inlineStr"/>
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr"/>
+      <c r="L5" s="2" t="inlineStr"/>
+      <c r="M5" s="2" t="inlineStr"/>
+      <c r="N5" s="2" t="inlineStr"/>
+      <c r="O5" s="2" t="inlineStr"/>
+      <c r="P5" s="2" t="inlineStr"/>
+      <c r="Q5" s="2" t="inlineStr"/>
+      <c r="R5" s="2" t="inlineStr"/>
+      <c r="S5" s="2" t="inlineStr"/>
+      <c r="T5" s="2" t="inlineStr"/>
+      <c r="U5" s="2" t="inlineStr"/>
+      <c r="V5" s="2" t="inlineStr"/>
+      <c r="W5" s="2" t="inlineStr"/>
+      <c r="X5" s="2" t="inlineStr"/>
+      <c r="Y5" s="2" t="inlineStr"/>
+      <c r="Z5" s="2" t="inlineStr"/>
+      <c r="AA5" s="2" t="inlineStr"/>
+      <c r="AB5" s="2" t="inlineStr"/>
+      <c r="AC5" s="2" t="inlineStr"/>
+      <c r="AD5" s="2" t="inlineStr"/>
+      <c r="AE5" s="2" t="inlineStr"/>
+      <c r="AF5" s="2" t="inlineStr">
+        <is>
+          <t>玄孙女曝光我的仙人身份藏不住了</t>
+        </is>
+      </c>
+      <c r="AG5" s="2" t="inlineStr">
+        <is>
+          <t>全球淹没我打造出了一座城池</t>
+        </is>
+      </c>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>我家浴缸通海底</t>
+        </is>
+      </c>
+      <c r="AI5" s="2" t="inlineStr">
+        <is>
+          <t>分家后我靠聚宝镯走上人生巅峰</t>
+        </is>
+      </c>
+      <c r="AJ5" s="2" t="inlineStr">
+        <is>
+          <t>九龙归位震八方</t>
+        </is>
+      </c>
+      <c r="AK5" s="2" t="inlineStr">
+        <is>
+          <t>我相亲捡属性开局怒怼化债女</t>
+        </is>
+      </c>
+      <c r="AL5" s="2" t="inlineStr">
+        <is>
+          <t>满级枪神回都市开局领证</t>
+        </is>
+      </c>
+      <c r="AM5" s="2" t="inlineStr">
+        <is>
+          <t>全民荒原求生</t>
+        </is>
+      </c>
+      <c r="AN5" s="2" t="inlineStr">
+        <is>
+          <t>万古第一仙在都市</t>
+        </is>
+      </c>
+      <c r="AO5" s="2" t="inlineStr">
+        <is>
+          <t>水库无限加速钓鱼佬排队爆杆</t>
+        </is>
+      </c>
+      <c r="AP5" s="2" t="inlineStr">
+        <is>
+          <t>战神归来前妻你哭什么</t>
+        </is>
+      </c>
+      <c r="AQ5" s="2" t="inlineStr">
+        <is>
+          <t>旁人笑我木讷不知我有老仙金手指</t>
+        </is>
+      </c>
+      <c r="AR5" s="2" t="inlineStr">
+        <is>
+          <t>婚礼照常新娘换人</t>
+        </is>
+      </c>
+      <c r="AS5" s="2" t="inlineStr">
+        <is>
+          <t>穿越女频开局送皇后白月光进东厂</t>
+        </is>
+      </c>
+      <c r="AT5" s="2" t="inlineStr">
+        <is>
+          <t>龙神报恩我一出海鱼获满满</t>
+        </is>
+      </c>
+      <c r="AU5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AW5" s="2" t="inlineStr"/>
+      <c r="AX5" s="2" t="inlineStr"/>
+      <c r="AY5" s="2" t="inlineStr"/>
+      <c r="AZ5" s="2" t="inlineStr">
+        <is>
+          <t>我在豪门装穷的日子/</t>
+        </is>
+      </c>
+      <c r="BA5" s="2" t="inlineStr">
+        <is>
+          <t>九世仙帝：王者归来</t>
+        </is>
+      </c>
+      <c r="BB5" s="2" t="inlineStr">
+        <is>
+          <t>我仙途陨落，唯宠一人</t>
+        </is>
+      </c>
+      <c r="BC5" s="2" t="inlineStr">
+        <is>
+          <t>战神隐世：我的傲娇总裁表妹</t>
+        </is>
+      </c>
+      <c r="BD5" s="2" t="inlineStr">
+        <is>
+          <t>娱乐圈凶神：我演反派就续命！</t>
+        </is>
+      </c>
+      <c r="BE5" s="2" t="inlineStr"/>
+      <c r="BF5" s="2" t="inlineStr"/>
+      <c r="BG5" s="2" t="inlineStr"/>
+      <c r="BH5" s="2" t="inlineStr"/>
+      <c r="BI5" s="2" t="inlineStr"/>
+      <c r="BJ5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6" ht="100" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>片源条件</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>最新资源表“最新剧集”：男频、菲律宾语标有或有/新；同剧任何版本文字标禁播或代运营则排除。按用户既定要求仅核验文字标记，不据颜色推断。</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="48" customHeight="1">
+          <t>俄语男频</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr"/>
+      <c r="C6" s="2" t="inlineStr"/>
+      <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr"/>
+      <c r="N6" s="2" t="inlineStr"/>
+      <c r="O6" s="2" t="inlineStr"/>
+      <c r="P6" s="2" t="inlineStr"/>
+      <c r="Q6" s="2" t="inlineStr"/>
+      <c r="R6" s="2" t="inlineStr"/>
+      <c r="S6" s="2" t="inlineStr"/>
+      <c r="T6" s="2" t="inlineStr"/>
+      <c r="U6" s="2" t="inlineStr"/>
+      <c r="V6" s="2" t="inlineStr"/>
+      <c r="W6" s="2" t="inlineStr"/>
+      <c r="X6" s="2" t="inlineStr"/>
+      <c r="Y6" s="2" t="inlineStr"/>
+      <c r="Z6" s="2" t="inlineStr"/>
+      <c r="AA6" s="2" t="inlineStr"/>
+      <c r="AB6" s="2" t="inlineStr"/>
+      <c r="AC6" s="2" t="inlineStr"/>
+      <c r="AD6" s="2" t="inlineStr"/>
+      <c r="AE6" s="2" t="inlineStr"/>
+      <c r="AF6" s="2" t="inlineStr"/>
+      <c r="AG6" s="2" t="inlineStr"/>
+      <c r="AH6" s="2" t="inlineStr"/>
+      <c r="AI6" s="2" t="inlineStr"/>
+      <c r="AJ6" s="2" t="inlineStr">
+        <is>
+          <t>边疆老卒御赐老婆后我越活越勇</t>
+        </is>
+      </c>
+      <c r="AK6" s="2" t="inlineStr">
+        <is>
+          <t>我宗门真的全是老弱病残啊</t>
+        </is>
+      </c>
+      <c r="AL6" s="2" t="inlineStr">
+        <is>
+          <t>我靠医术横扫江都</t>
+        </is>
+      </c>
+      <c r="AM6" s="2" t="inlineStr">
+        <is>
+          <t>武魂觉醒我用锤子一人成军</t>
+        </is>
+      </c>
+      <c r="AN6" s="2" t="inlineStr">
+        <is>
+          <t>九龙归位震八方</t>
+        </is>
+      </c>
+      <c r="AO6" s="2" t="inlineStr">
+        <is>
+          <t>分家后我靠聚宝镯走上人生巅峰</t>
+        </is>
+      </c>
+      <c r="AP6" s="2" t="inlineStr">
+        <is>
+          <t>我相亲捡属性开局怒怼化债女</t>
+        </is>
+      </c>
+      <c r="AQ6" s="2" t="inlineStr">
+        <is>
+          <t>归来后我踩碎所有偏见</t>
+        </is>
+      </c>
+      <c r="AR6" s="2" t="inlineStr">
+        <is>
+          <t>战神归来前妻你哭什么</t>
+        </is>
+      </c>
+      <c r="AS6" s="2" t="inlineStr">
+        <is>
+          <t>旁人笑我木讷不知我有老仙金手指</t>
+        </is>
+      </c>
+      <c r="AT6" s="2" t="inlineStr">
+        <is>
+          <t>婚礼照常新娘换人</t>
+        </is>
+      </c>
+      <c r="AU6" s="2" t="inlineStr">
+        <is>
+          <t>穿越女频开局送皇后白月光进东厂</t>
+        </is>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>龙神报恩我一出海鱼获满满</t>
+        </is>
+      </c>
+      <c r="AW6" s="2" t="inlineStr">
+        <is>
+          <t>我造的机甲被老婆直播曝光了</t>
+        </is>
+      </c>
+      <c r="AX6" s="2" t="inlineStr">
+        <is>
+          <t>猴王报恩全村傻眼了</t>
+        </is>
+      </c>
+      <c r="AY6" s="2" t="inlineStr">
+        <is>
+          <t>我家浴缸通海底</t>
+        </is>
+      </c>
+      <c r="AZ6" s="2" t="inlineStr">
+        <is>
+          <t>玄孙女曝光我的仙人身份藏不住了</t>
+        </is>
+      </c>
+      <c r="BA6" s="2" t="inlineStr">
+        <is>
+          <t>渔夫从神奇龙珠开始起飞</t>
+        </is>
+      </c>
+      <c r="BB6" s="2" t="inlineStr">
+        <is>
+          <t>万倍返还弟子越强我越神</t>
+        </is>
+      </c>
+      <c r="BC6" s="2" t="inlineStr">
+        <is>
+          <t>满级大师兄制霸都市</t>
+        </is>
+      </c>
+      <c r="BD6" s="2" t="inlineStr">
+        <is>
+          <t>囤千万物资到古代娶女帝</t>
+        </is>
+      </c>
+      <c r="BE6" s="2" t="inlineStr">
+        <is>
+          <t>跌入古井觉醒神农秘术</t>
+        </is>
+      </c>
+      <c r="BF6" s="2" t="inlineStr"/>
+      <c r="BG6" s="2" t="inlineStr"/>
+      <c r="BH6" s="2" t="inlineStr"/>
+      <c r="BI6" s="2" t="inlineStr"/>
+      <c r="BJ6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7" ht="100" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026年份依据</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>本次22部均为2026 WW代码片源，资源表未填明确出剧日期。仅确认代码标2026年，不将代码年份当作具体出剧日期或最新月份。</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="48" customHeight="1">
+          <t>英语男频2</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr"/>
+      <c r="C7" s="2" t="inlineStr"/>
+      <c r="D7" s="2" t="inlineStr"/>
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr"/>
+      <c r="K7" s="2" t="inlineStr"/>
+      <c r="L7" s="2" t="inlineStr"/>
+      <c r="M7" s="2" t="inlineStr"/>
+      <c r="N7" s="2" t="inlineStr"/>
+      <c r="O7" s="2" t="inlineStr"/>
+      <c r="P7" s="2" t="inlineStr"/>
+      <c r="Q7" s="2" t="inlineStr"/>
+      <c r="R7" s="2" t="inlineStr"/>
+      <c r="S7" s="2" t="inlineStr"/>
+      <c r="T7" s="2" t="inlineStr"/>
+      <c r="U7" s="2" t="inlineStr"/>
+      <c r="V7" s="2" t="inlineStr"/>
+      <c r="W7" s="2" t="inlineStr"/>
+      <c r="X7" s="2" t="inlineStr"/>
+      <c r="Y7" s="2" t="inlineStr"/>
+      <c r="Z7" s="2" t="inlineStr"/>
+      <c r="AA7" s="2" t="inlineStr"/>
+      <c r="AB7" s="2" t="inlineStr"/>
+      <c r="AC7" s="2" t="inlineStr"/>
+      <c r="AD7" s="2" t="inlineStr"/>
+      <c r="AE7" s="2" t="inlineStr"/>
+      <c r="AF7" s="2" t="inlineStr"/>
+      <c r="AG7" s="2" t="inlineStr"/>
+      <c r="AH7" s="2" t="inlineStr"/>
+      <c r="AI7" s="2" t="inlineStr"/>
+      <c r="AJ7" s="2" t="inlineStr"/>
+      <c r="AK7" s="2" t="inlineStr"/>
+      <c r="AL7" s="2" t="inlineStr"/>
+      <c r="AM7" s="2" t="inlineStr"/>
+      <c r="AN7" s="2" t="inlineStr">
+        <is>
+          <t>神临我自执剑迎</t>
+        </is>
+      </c>
+      <c r="AO7" s="2" t="inlineStr">
+        <is>
+          <t>分家开出海神的鱼钩</t>
+        </is>
+      </c>
+      <c r="AP7" s="2" t="inlineStr">
+        <is>
+          <t>满级大师兄制霸都市</t>
+        </is>
+      </c>
+      <c r="AQ7" s="2" t="inlineStr">
+        <is>
+          <t>满朝文武都是我兄弟</t>
+        </is>
+      </c>
+      <c r="AR7" s="2" t="inlineStr">
+        <is>
+          <t>开局流放我用系统搬空皇帝库房</t>
+        </is>
+      </c>
+      <c r="AS7" s="2" t="inlineStr">
+        <is>
+          <t>是谁坑惨了朕</t>
+        </is>
+      </c>
+      <c r="AT7" s="2" t="inlineStr">
+        <is>
+          <t>我真是昏君你们快造反吧</t>
+        </is>
+      </c>
+      <c r="AU7" s="2" t="inlineStr">
+        <is>
+          <t>我用科技征服人皇</t>
+        </is>
+      </c>
+      <c r="AV7" s="2" t="inlineStr">
+        <is>
+          <t>全球淹没我打造出了一座城池</t>
+        </is>
+      </c>
+      <c r="AW7" s="2" t="inlineStr">
+        <is>
+          <t>囤千万物资到古代娶女帝</t>
+        </is>
+      </c>
+      <c r="AX7" s="2" t="inlineStr">
+        <is>
+          <t>龙皇归来：不想当战神只要宠女儿</t>
+        </is>
+      </c>
+      <c r="AY7" s="2" t="inlineStr">
+        <is>
+          <t>流放开局，我卷走皇帝的小金库2</t>
+        </is>
+      </c>
+      <c r="AZ7" s="2" t="inlineStr">
+        <is>
+          <t>开局成破剑竟被她进化成神兵</t>
+        </is>
+      </c>
+      <c r="BA7" s="2" t="inlineStr">
+        <is>
+          <t>代号枪神</t>
+        </is>
+      </c>
+      <c r="BB7" s="2" t="inlineStr"/>
+      <c r="BC7" s="2" t="inlineStr"/>
+      <c r="BD7" s="2" t="inlineStr"/>
+      <c r="BE7" s="2" t="inlineStr"/>
+      <c r="BF7" s="2" t="inlineStr"/>
+      <c r="BG7" s="2" t="inlineStr"/>
+      <c r="BH7" s="2" t="inlineStr"/>
+      <c r="BI7" s="2" t="inlineStr"/>
+      <c r="BJ7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8" ht="100" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>外采解禁慢</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>11部标注“外采剧-解禁慢”，其中5部为原有安排、6部新增。未标禁播不代表已获版权放行，发布前按实际Studio版权状态核对；排期表已保留该状态。</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="48" customHeight="1">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>历史去重</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>新增17部与上传菲律宾语历史及此前已交付片单不重复；22部内部剧名和代码均无重复。</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="48" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>同剧错峰</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>新增剧与本次其他频道表及已知未覆盖后续排片至少168小时；只给日期的按全天区间保守计算。命中无日期记录的候选不安排。</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="48" customHeight="1">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>交付范围</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>仅生成排片Excel、CSV和JSON，未修改线上飞书、YouTube或程序素材；未核验实际视频音轨。已有素材、标题和旧程序均不改。</t>
-        </is>
-      </c>
+          <t>（注：部分内容由豆包工作 AI 生成）</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr"/>
+      <c r="C8" s="2" t="inlineStr"/>
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="inlineStr"/>
+      <c r="N8" s="2" t="inlineStr"/>
+      <c r="O8" s="2" t="inlineStr"/>
+      <c r="P8" s="2" t="inlineStr"/>
+      <c r="Q8" s="2" t="inlineStr"/>
+      <c r="R8" s="2" t="inlineStr"/>
+      <c r="S8" s="2" t="inlineStr"/>
+      <c r="T8" s="2" t="inlineStr"/>
+      <c r="U8" s="2" t="inlineStr"/>
+      <c r="V8" s="2" t="inlineStr"/>
+      <c r="W8" s="2" t="inlineStr"/>
+      <c r="X8" s="2" t="inlineStr"/>
+      <c r="Y8" s="2" t="inlineStr"/>
+      <c r="Z8" s="2" t="inlineStr"/>
+      <c r="AA8" s="2" t="inlineStr"/>
+      <c r="AB8" s="2" t="inlineStr"/>
+      <c r="AC8" s="2" t="inlineStr"/>
+      <c r="AD8" s="2" t="inlineStr"/>
+      <c r="AE8" s="2" t="inlineStr"/>
+      <c r="AF8" s="2" t="inlineStr"/>
+      <c r="AG8" s="2" t="inlineStr"/>
+      <c r="AH8" s="2" t="inlineStr"/>
+      <c r="AI8" s="2" t="inlineStr"/>
+      <c r="AJ8" s="2" t="inlineStr"/>
+      <c r="AK8" s="2" t="inlineStr"/>
+      <c r="AL8" s="2" t="inlineStr"/>
+      <c r="AM8" s="2" t="inlineStr"/>
+      <c r="AN8" s="2" t="inlineStr"/>
+      <c r="AO8" s="2" t="inlineStr"/>
+      <c r="AP8" s="2" t="inlineStr"/>
+      <c r="AQ8" s="2" t="inlineStr"/>
+      <c r="AR8" s="2" t="inlineStr"/>
+      <c r="AS8" s="2" t="inlineStr"/>
+      <c r="AT8" s="2" t="inlineStr"/>
+      <c r="AU8" s="2" t="inlineStr"/>
+      <c r="AV8" s="2" t="inlineStr"/>
+      <c r="AW8" s="2" t="inlineStr"/>
+      <c r="AX8" s="2" t="inlineStr"/>
+      <c r="AY8" s="2" t="inlineStr"/>
+      <c r="AZ8" s="2" t="inlineStr"/>
+      <c r="BA8" s="2" t="inlineStr"/>
+      <c r="BB8" s="2" t="inlineStr"/>
+      <c r="BC8" s="2" t="inlineStr"/>
+      <c r="BD8" s="2" t="inlineStr"/>
+      <c r="BE8" s="2" t="inlineStr"/>
+      <c r="BF8" s="2" t="inlineStr"/>
+      <c r="BG8" s="2" t="inlineStr"/>
+      <c r="BH8" s="2" t="inlineStr"/>
+      <c r="BI8" s="2" t="inlineStr"/>
+      <c r="BJ8" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>